<commit_message>
Improve financial template guidance
</commit_message>
<xml_diff>
--- a/docs/templates/elidan-financial-template-v2.xlsx
+++ b/docs/templates/elidan-financial-template-v2.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R1056edc2dade444c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Cash" sheetId="2" r:id="R3a830df9e96d4ee2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Optional Detail" sheetId="3" r:id="R3fa45b34fd8c448a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worked Example" sheetId="4" r:id="R83778716cd3a4b63"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Start Here" sheetId="1" r:id="R7330aaf599344b65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Monthly Cash" sheetId="2" r:id="R37d1e28557114c78"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Optional Detail" sheetId="3" r:id="Rfd11a14c62354dca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Worked Example" sheetId="4" r:id="R48a16da31f12427a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -16,13 +16,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="4">
+  <x:numFmts count="5">
     <x:numFmt numFmtId="200" formatCode="0"/>
     <x:numFmt numFmtId="201" formatCode="mmm-yy"/>
     <x:numFmt numFmtId="202" formatCode="dd-mmm-yy"/>
     <x:numFmt numFmtId="203" formatCode="#,##0;[Red](#,##0);-"/>
+    <x:numFmt numFmtId="204" formatCode="$#,##0.00;[Red]-$#,##0.00;$0.00"/>
   </x:numFmts>
-  <x:fonts count="10">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -78,8 +79,38 @@
       <x:color rgb="FF243B53"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF20334D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF20334D"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF20334D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF20334D"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="9">
+  <x:fills count="12">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -119,6 +150,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFEEF2F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE9EEF3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2AA7A1"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF2AA7A1"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -375,7 +421,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="101">
+  <x:cellXfs count="133">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -533,6 +579,82 @@
     <x:xf numFmtId="203" fontId="9" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="203" fontId="9" fillId="8" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="9" fillId="8" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="9" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="203" fontId="9" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="9" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="9" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="204" fontId="9" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="204" fontId="9" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -544,7 +666,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -555,7 +677,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -566,7 +688,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -577,7 +699,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -588,7 +710,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -599,7 +721,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -610,7 +732,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -621,7 +743,7 @@
         <x:color rgb="FFB42318"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDECEC"/>
         </x:patternFill>
       </x:fill>
@@ -878,7 +1000,7 @@
     </x:row>
     <x:row r="3" ht="30" customHeight="1">
       <x:c r="A3" s="7" t="str">
-        <x:v>Version 2.0  |  Enter completed monthly cash activity. The workbook checks whether cash changes reconcile before upload.</x:v>
+        <x:v>Version 2.1  |  Enter completed monthly cash activity. Built-in checks compare actual cash with the activity you enter.</x:v>
       </x:c>
       <x:c r="B3" s="7" t="str">
         <x:v>Version 2.0  |  Enter completed monthly cash activity. The workbook checks whether cash changes reconcile before upload.</x:v>
@@ -1072,29 +1194,41 @@
       <x:c r="E19" s="22"/>
       <x:c r="F19" s="22"/>
     </x:row>
-    <x:row r="20" ht="32" customHeight="1">
-      <x:c r="A20" s="13" t="str">
-        <x:v>Check the difference</x:v>
-      </x:c>
-      <x:c r="B20" s="22" t="str">
-        <x:v>A reconciliation difference near zero means the entered cash activity explains the change from opening to closing cash.</x:v>
-      </x:c>
-      <x:c r="C20" s="22"/>
-      <x:c r="D20" s="22"/>
-      <x:c r="E20" s="22"/>
-      <x:c r="F20" s="22"/>
-    </x:row>
-    <x:row r="21" ht="32" customHeight="1">
-      <x:c r="A21" s="13" t="str">
+    <x:row r="20" ht="48" customHeight="1">
+      <x:c r="A20" s="119" t="str">
+        <x:v>Compare expected and actual cash</x:v>
+      </x:c>
+      <x:c r="B20" s="120" t="str">
+        <x:v>Expected closing cash is calculated from opening cash and monthly activity. Enter actual closing cash from your bank or accounting records; do not replace it with the calculated amount.</x:v>
+      </x:c>
+      <x:c r="C20" s="120"/>
+      <x:c r="D20" s="120"/>
+      <x:c r="E20" s="120"/>
+      <x:c r="F20" s="120"/>
+    </x:row>
+    <x:row r="21" ht="48" customHeight="1">
+      <x:c r="A21" s="119" t="str">
+        <x:v>Confirm opening cash</x:v>
+      </x:c>
+      <x:c r="B21" s="120" t="str">
+        <x:v>For each consecutive month, review the opening balance check. Copy the prior closing balance only after confirming it matches the next month's actual opening balance.</x:v>
+      </x:c>
+      <x:c r="C21" s="120"/>
+      <x:c r="D21" s="120"/>
+      <x:c r="E21" s="120"/>
+      <x:c r="F21" s="120"/>
+    </x:row>
+    <x:row r="22" ht="42" customHeight="1">
+      <x:c r="A22" s="122" t="str">
         <x:v>Optional context</x:v>
       </x:c>
-      <x:c r="B21" s="22" t="str">
+      <x:c r="B22" s="123" t="str">
         <x:v>Use Optional Detail for reserved taxes, near-term receivables and bills, credit availability, and the lowest observed cash balance.</x:v>
       </x:c>
-      <x:c r="C21" s="22"/>
-      <x:c r="D21" s="22"/>
-      <x:c r="E21" s="22"/>
-      <x:c r="F21" s="22"/>
+      <x:c r="C22" s="123"/>
+      <x:c r="D22" s="123"/>
+      <x:c r="E22" s="123"/>
+      <x:c r="F22" s="123"/>
     </x:row>
     <x:row r="23" ht="22" customHeight="1">
       <x:c r="A23" s="10" t="str">
@@ -1215,14 +1349,15 @@
     <x:mergeCell ref="B17:F17"/>
     <x:mergeCell ref="B18:F18"/>
     <x:mergeCell ref="B19:F19"/>
-    <x:mergeCell ref="B20:F20"/>
-    <x:mergeCell ref="B21:F21"/>
     <x:mergeCell ref="A23:F23"/>
     <x:mergeCell ref="B24:F24"/>
     <x:mergeCell ref="B25:F25"/>
     <x:mergeCell ref="B26:F26"/>
     <x:mergeCell ref="B27:F27"/>
     <x:mergeCell ref="A29:F30"/>
+    <x:mergeCell ref="B20:F20"/>
+    <x:mergeCell ref="B21:F21"/>
+    <x:mergeCell ref="B22:F22"/>
   </x:mergeCells>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="B12">
@@ -1257,9 +1392,11 @@
     <x:col min="15" max="15" width="17" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="17" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="17" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="18" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="24" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="28" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="24" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="25" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -1509,6 +1646,9 @@
       <x:c r="T5" s="45" t="str">
         <x:v>NOTES</x:v>
       </x:c>
+      <x:c r="V5" s="117" t="str">
+        <x:v>NOTES</x:v>
+      </x:c>
     </x:row>
     <x:row r="6" ht="46" customHeight="1">
       <x:c r="A6" s="51" t="str">
@@ -1563,12 +1703,18 @@
         <x:v>Unavailable cash</x:v>
       </x:c>
       <x:c r="R6" s="51" t="str">
+        <x:v>Expected closing cash</x:v>
+      </x:c>
+      <x:c r="S6" s="51" t="str">
         <x:v>Reconciliation difference</x:v>
       </x:c>
-      <x:c r="S6" s="51" t="str">
+      <x:c r="T6" s="51" t="str">
+        <x:v>Opening balance check</x:v>
+      </x:c>
+      <x:c r="U6" s="51" t="str">
         <x:v>Row check</x:v>
       </x:c>
-      <x:c r="T6" s="51" t="str">
+      <x:c r="V6" s="51" t="str">
         <x:v>Notes</x:v>
       </x:c>
     </x:row>
@@ -1590,13 +1736,19 @@
       <x:c r="O7" s="64"/>
       <x:c r="P7" s="64"/>
       <x:c r="Q7" s="64"/>
-      <x:c r="R7" s="65" t="str">
-        <x:f>IF($A7="","",IF(COUNT($D7:$Q7)&lt;14,"",ROUND($P7-$D7-($E7-$F7-$G7-$H7-$I7-$J7+$K7+$L7+$M7+$N7-$O7),2)))</x:f>
-      </x:c>
-      <x:c r="S7" s="58" t="str">
-        <x:f>IF($A7="","",IF(DAY($A7)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A7)&gt;1,"Duplicate month",IF(OR($B7="",COUNT($D7:$Q7)&lt;14),"Complete required cells",IF($Q7&gt;MAX($P7,0),"Unavailable cash exceeds closing cash",IF($B7="Partial",IF($C7="","Add cutoff date",IF(OR(YEAR($C7)&lt;&gt;YEAR($A7),MONTH($C7)&lt;&gt;MONTH($A7)),"Cutoff must be in month",IF(ABS($R7)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C7&lt;&gt;"","Remove cutoff date",IF(ABS($R7)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T7" s="54"/>
+      <x:c r="R7" s="107" t="str">
+        <x:f>IF($A7="","",IF(COUNT($D7:$O7)&lt;12,"",ROUND($D7+$E7-$F7-$G7-$H7-$I7-$J7+$K7+$L7+$M7+$N7-$O7,2)))</x:f>
+      </x:c>
+      <x:c r="S7" s="107" t="str">
+        <x:f>IF($A7="","",IF(OR($P7="",$R7=""),"",ROUND($P7-$R7,2)))</x:f>
+      </x:c>
+      <x:c r="T7" s="108" t="str">
+        <x:f>IF($A7="","","First entered month")</x:f>
+      </x:c>
+      <x:c r="U7" s="108" t="str">
+        <x:f>IF($A7="","",IF(DAY($A7)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A7)&gt;1,"Duplicate month",IF(OR($B7="",COUNT($D7:$Q7)&lt;14),"Complete required cells",IF($Q7&gt;MAX($P7,0),"Unavailable cash exceeds closing cash",IF($B7="Partial",IF($C7="","Add cutoff date",IF(OR(YEAR($C7)&lt;&gt;YEAR($A7),MONTH($C7)&lt;&gt;MONTH($A7)),"Cutoff must be in month",IF(ABS($S7)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C7&lt;&gt;"","Remove cutoff date",IF(ABS($S7)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V7" s="54"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="61"/>
@@ -1616,13 +1768,19 @@
       <x:c r="O8" s="66"/>
       <x:c r="P8" s="66"/>
       <x:c r="Q8" s="66"/>
-      <x:c r="R8" s="67" t="str">
-        <x:f>IF($A8="","",IF(COUNT($D8:$Q8)&lt;14,"",ROUND($P8-$D8-($E8-$F8-$G8-$H8-$I8-$J8+$K8+$L8+$M8+$N8-$O8),2)))</x:f>
-      </x:c>
-      <x:c r="S8" s="59" t="str">
-        <x:f>IF($A8="","",IF(DAY($A8)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A8)&gt;1,"Duplicate month",IF(OR($B8="",COUNT($D8:$Q8)&lt;14),"Complete required cells",IF($Q8&gt;MAX($P8,0),"Unavailable cash exceeds closing cash",IF($B8="Partial",IF($C8="","Add cutoff date",IF(OR(YEAR($C8)&lt;&gt;YEAR($A8),MONTH($C8)&lt;&gt;MONTH($A8)),"Cutoff must be in month",IF(ABS($R8)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C8&lt;&gt;"","Remove cutoff date",IF(ABS($R8)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T8" s="55"/>
+      <x:c r="R8" s="109" t="str">
+        <x:f>IF($A8="","",IF(COUNT($D8:$O8)&lt;12,"",ROUND($D8+$E8-$F8-$G8-$H8-$I8-$J8+$K8+$L8+$M8+$N8-$O8,2)))</x:f>
+      </x:c>
+      <x:c r="S8" s="109" t="str">
+        <x:f>IF($A8="","",IF(OR($P8="",$R8=""),"",ROUND($P8-$R8,2)))</x:f>
+      </x:c>
+      <x:c r="T8" s="110" t="str">
+        <x:f>IF($A8="","",IF($A7="","No prior row to compare",IF(EDATE($A7,1)&lt;&gt;$A8,"Check month sequence",IF(OR($D8="",$P7=""),"Check opening cash",IF(ABS($D8-$P7)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U8" s="110" t="str">
+        <x:f>IF($A8="","",IF(DAY($A8)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A8)&gt;1,"Duplicate month",IF(OR($B8="",COUNT($D8:$Q8)&lt;14),"Complete required cells",IF($Q8&gt;MAX($P8,0),"Unavailable cash exceeds closing cash",IF($B8="Partial",IF($C8="","Add cutoff date",IF(OR(YEAR($C8)&lt;&gt;YEAR($A8),MONTH($C8)&lt;&gt;MONTH($A8)),"Cutoff must be in month",IF(ABS($S8)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C8&lt;&gt;"","Remove cutoff date",IF(ABS($S8)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V8" s="55"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="61"/>
@@ -1642,13 +1800,19 @@
       <x:c r="O9" s="66"/>
       <x:c r="P9" s="66"/>
       <x:c r="Q9" s="66"/>
-      <x:c r="R9" s="67" t="str">
-        <x:f>IF($A9="","",IF(COUNT($D9:$Q9)&lt;14,"",ROUND($P9-$D9-($E9-$F9-$G9-$H9-$I9-$J9+$K9+$L9+$M9+$N9-$O9),2)))</x:f>
-      </x:c>
-      <x:c r="S9" s="59" t="str">
-        <x:f>IF($A9="","",IF(DAY($A9)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A9)&gt;1,"Duplicate month",IF(OR($B9="",COUNT($D9:$Q9)&lt;14),"Complete required cells",IF($Q9&gt;MAX($P9,0),"Unavailable cash exceeds closing cash",IF($B9="Partial",IF($C9="","Add cutoff date",IF(OR(YEAR($C9)&lt;&gt;YEAR($A9),MONTH($C9)&lt;&gt;MONTH($A9)),"Cutoff must be in month",IF(ABS($R9)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C9&lt;&gt;"","Remove cutoff date",IF(ABS($R9)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T9" s="55"/>
+      <x:c r="R9" s="109" t="str">
+        <x:f>IF($A9="","",IF(COUNT($D9:$O9)&lt;12,"",ROUND($D9+$E9-$F9-$G9-$H9-$I9-$J9+$K9+$L9+$M9+$N9-$O9,2)))</x:f>
+      </x:c>
+      <x:c r="S9" s="109" t="str">
+        <x:f>IF($A9="","",IF(OR($P9="",$R9=""),"",ROUND($P9-$R9,2)))</x:f>
+      </x:c>
+      <x:c r="T9" s="110" t="str">
+        <x:f>IF($A9="","",IF($A8="","No prior row to compare",IF(EDATE($A8,1)&lt;&gt;$A9,"Check month sequence",IF(OR($D9="",$P8=""),"Check opening cash",IF(ABS($D9-$P8)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U9" s="110" t="str">
+        <x:f>IF($A9="","",IF(DAY($A9)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A9)&gt;1,"Duplicate month",IF(OR($B9="",COUNT($D9:$Q9)&lt;14),"Complete required cells",IF($Q9&gt;MAX($P9,0),"Unavailable cash exceeds closing cash",IF($B9="Partial",IF($C9="","Add cutoff date",IF(OR(YEAR($C9)&lt;&gt;YEAR($A9),MONTH($C9)&lt;&gt;MONTH($A9)),"Cutoff must be in month",IF(ABS($S9)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C9&lt;&gt;"","Remove cutoff date",IF(ABS($S9)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V9" s="55"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="61"/>
@@ -1668,13 +1832,19 @@
       <x:c r="O10" s="66"/>
       <x:c r="P10" s="66"/>
       <x:c r="Q10" s="66"/>
-      <x:c r="R10" s="67" t="str">
-        <x:f>IF($A10="","",IF(COUNT($D10:$Q10)&lt;14,"",ROUND($P10-$D10-($E10-$F10-$G10-$H10-$I10-$J10+$K10+$L10+$M10+$N10-$O10),2)))</x:f>
-      </x:c>
-      <x:c r="S10" s="59" t="str">
-        <x:f>IF($A10="","",IF(DAY($A10)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A10)&gt;1,"Duplicate month",IF(OR($B10="",COUNT($D10:$Q10)&lt;14),"Complete required cells",IF($Q10&gt;MAX($P10,0),"Unavailable cash exceeds closing cash",IF($B10="Partial",IF($C10="","Add cutoff date",IF(OR(YEAR($C10)&lt;&gt;YEAR($A10),MONTH($C10)&lt;&gt;MONTH($A10)),"Cutoff must be in month",IF(ABS($R10)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C10&lt;&gt;"","Remove cutoff date",IF(ABS($R10)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T10" s="55"/>
+      <x:c r="R10" s="109" t="str">
+        <x:f>IF($A10="","",IF(COUNT($D10:$O10)&lt;12,"",ROUND($D10+$E10-$F10-$G10-$H10-$I10-$J10+$K10+$L10+$M10+$N10-$O10,2)))</x:f>
+      </x:c>
+      <x:c r="S10" s="109" t="str">
+        <x:f>IF($A10="","",IF(OR($P10="",$R10=""),"",ROUND($P10-$R10,2)))</x:f>
+      </x:c>
+      <x:c r="T10" s="110" t="str">
+        <x:f>IF($A10="","",IF($A9="","No prior row to compare",IF(EDATE($A9,1)&lt;&gt;$A10,"Check month sequence",IF(OR($D10="",$P9=""),"Check opening cash",IF(ABS($D10-$P9)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U10" s="110" t="str">
+        <x:f>IF($A10="","",IF(DAY($A10)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A10)&gt;1,"Duplicate month",IF(OR($B10="",COUNT($D10:$Q10)&lt;14),"Complete required cells",IF($Q10&gt;MAX($P10,0),"Unavailable cash exceeds closing cash",IF($B10="Partial",IF($C10="","Add cutoff date",IF(OR(YEAR($C10)&lt;&gt;YEAR($A10),MONTH($C10)&lt;&gt;MONTH($A10)),"Cutoff must be in month",IF(ABS($S10)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C10&lt;&gt;"","Remove cutoff date",IF(ABS($S10)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V10" s="55"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="61"/>
@@ -1694,13 +1864,19 @@
       <x:c r="O11" s="66"/>
       <x:c r="P11" s="66"/>
       <x:c r="Q11" s="66"/>
-      <x:c r="R11" s="67" t="str">
-        <x:f>IF($A11="","",IF(COUNT($D11:$Q11)&lt;14,"",ROUND($P11-$D11-($E11-$F11-$G11-$H11-$I11-$J11+$K11+$L11+$M11+$N11-$O11),2)))</x:f>
-      </x:c>
-      <x:c r="S11" s="59" t="str">
-        <x:f>IF($A11="","",IF(DAY($A11)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A11)&gt;1,"Duplicate month",IF(OR($B11="",COUNT($D11:$Q11)&lt;14),"Complete required cells",IF($Q11&gt;MAX($P11,0),"Unavailable cash exceeds closing cash",IF($B11="Partial",IF($C11="","Add cutoff date",IF(OR(YEAR($C11)&lt;&gt;YEAR($A11),MONTH($C11)&lt;&gt;MONTH($A11)),"Cutoff must be in month",IF(ABS($R11)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C11&lt;&gt;"","Remove cutoff date",IF(ABS($R11)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T11" s="55"/>
+      <x:c r="R11" s="109" t="str">
+        <x:f>IF($A11="","",IF(COUNT($D11:$O11)&lt;12,"",ROUND($D11+$E11-$F11-$G11-$H11-$I11-$J11+$K11+$L11+$M11+$N11-$O11,2)))</x:f>
+      </x:c>
+      <x:c r="S11" s="109" t="str">
+        <x:f>IF($A11="","",IF(OR($P11="",$R11=""),"",ROUND($P11-$R11,2)))</x:f>
+      </x:c>
+      <x:c r="T11" s="110" t="str">
+        <x:f>IF($A11="","",IF($A10="","No prior row to compare",IF(EDATE($A10,1)&lt;&gt;$A11,"Check month sequence",IF(OR($D11="",$P10=""),"Check opening cash",IF(ABS($D11-$P10)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U11" s="110" t="str">
+        <x:f>IF($A11="","",IF(DAY($A11)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A11)&gt;1,"Duplicate month",IF(OR($B11="",COUNT($D11:$Q11)&lt;14),"Complete required cells",IF($Q11&gt;MAX($P11,0),"Unavailable cash exceeds closing cash",IF($B11="Partial",IF($C11="","Add cutoff date",IF(OR(YEAR($C11)&lt;&gt;YEAR($A11),MONTH($C11)&lt;&gt;MONTH($A11)),"Cutoff must be in month",IF(ABS($S11)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C11&lt;&gt;"","Remove cutoff date",IF(ABS($S11)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V11" s="55"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="61"/>
@@ -1720,13 +1896,19 @@
       <x:c r="O12" s="66"/>
       <x:c r="P12" s="66"/>
       <x:c r="Q12" s="66"/>
-      <x:c r="R12" s="67" t="str">
-        <x:f>IF($A12="","",IF(COUNT($D12:$Q12)&lt;14,"",ROUND($P12-$D12-($E12-$F12-$G12-$H12-$I12-$J12+$K12+$L12+$M12+$N12-$O12),2)))</x:f>
-      </x:c>
-      <x:c r="S12" s="59" t="str">
-        <x:f>IF($A12="","",IF(DAY($A12)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A12)&gt;1,"Duplicate month",IF(OR($B12="",COUNT($D12:$Q12)&lt;14),"Complete required cells",IF($Q12&gt;MAX($P12,0),"Unavailable cash exceeds closing cash",IF($B12="Partial",IF($C12="","Add cutoff date",IF(OR(YEAR($C12)&lt;&gt;YEAR($A12),MONTH($C12)&lt;&gt;MONTH($A12)),"Cutoff must be in month",IF(ABS($R12)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C12&lt;&gt;"","Remove cutoff date",IF(ABS($R12)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T12" s="55"/>
+      <x:c r="R12" s="109" t="str">
+        <x:f>IF($A12="","",IF(COUNT($D12:$O12)&lt;12,"",ROUND($D12+$E12-$F12-$G12-$H12-$I12-$J12+$K12+$L12+$M12+$N12-$O12,2)))</x:f>
+      </x:c>
+      <x:c r="S12" s="109" t="str">
+        <x:f>IF($A12="","",IF(OR($P12="",$R12=""),"",ROUND($P12-$R12,2)))</x:f>
+      </x:c>
+      <x:c r="T12" s="110" t="str">
+        <x:f>IF($A12="","",IF($A11="","No prior row to compare",IF(EDATE($A11,1)&lt;&gt;$A12,"Check month sequence",IF(OR($D12="",$P11=""),"Check opening cash",IF(ABS($D12-$P11)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U12" s="110" t="str">
+        <x:f>IF($A12="","",IF(DAY($A12)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A12)&gt;1,"Duplicate month",IF(OR($B12="",COUNT($D12:$Q12)&lt;14),"Complete required cells",IF($Q12&gt;MAX($P12,0),"Unavailable cash exceeds closing cash",IF($B12="Partial",IF($C12="","Add cutoff date",IF(OR(YEAR($C12)&lt;&gt;YEAR($A12),MONTH($C12)&lt;&gt;MONTH($A12)),"Cutoff must be in month",IF(ABS($S12)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C12&lt;&gt;"","Remove cutoff date",IF(ABS($S12)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V12" s="55"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="61"/>
@@ -1746,13 +1928,19 @@
       <x:c r="O13" s="66"/>
       <x:c r="P13" s="66"/>
       <x:c r="Q13" s="66"/>
-      <x:c r="R13" s="67" t="str">
-        <x:f>IF($A13="","",IF(COUNT($D13:$Q13)&lt;14,"",ROUND($P13-$D13-($E13-$F13-$G13-$H13-$I13-$J13+$K13+$L13+$M13+$N13-$O13),2)))</x:f>
-      </x:c>
-      <x:c r="S13" s="59" t="str">
-        <x:f>IF($A13="","",IF(DAY($A13)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A13)&gt;1,"Duplicate month",IF(OR($B13="",COUNT($D13:$Q13)&lt;14),"Complete required cells",IF($Q13&gt;MAX($P13,0),"Unavailable cash exceeds closing cash",IF($B13="Partial",IF($C13="","Add cutoff date",IF(OR(YEAR($C13)&lt;&gt;YEAR($A13),MONTH($C13)&lt;&gt;MONTH($A13)),"Cutoff must be in month",IF(ABS($R13)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C13&lt;&gt;"","Remove cutoff date",IF(ABS($R13)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T13" s="55"/>
+      <x:c r="R13" s="109" t="str">
+        <x:f>IF($A13="","",IF(COUNT($D13:$O13)&lt;12,"",ROUND($D13+$E13-$F13-$G13-$H13-$I13-$J13+$K13+$L13+$M13+$N13-$O13,2)))</x:f>
+      </x:c>
+      <x:c r="S13" s="109" t="str">
+        <x:f>IF($A13="","",IF(OR($P13="",$R13=""),"",ROUND($P13-$R13,2)))</x:f>
+      </x:c>
+      <x:c r="T13" s="110" t="str">
+        <x:f>IF($A13="","",IF($A12="","No prior row to compare",IF(EDATE($A12,1)&lt;&gt;$A13,"Check month sequence",IF(OR($D13="",$P12=""),"Check opening cash",IF(ABS($D13-$P12)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U13" s="110" t="str">
+        <x:f>IF($A13="","",IF(DAY($A13)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A13)&gt;1,"Duplicate month",IF(OR($B13="",COUNT($D13:$Q13)&lt;14),"Complete required cells",IF($Q13&gt;MAX($P13,0),"Unavailable cash exceeds closing cash",IF($B13="Partial",IF($C13="","Add cutoff date",IF(OR(YEAR($C13)&lt;&gt;YEAR($A13),MONTH($C13)&lt;&gt;MONTH($A13)),"Cutoff must be in month",IF(ABS($S13)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C13&lt;&gt;"","Remove cutoff date",IF(ABS($S13)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V13" s="55"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="61"/>
@@ -1772,13 +1960,19 @@
       <x:c r="O14" s="66"/>
       <x:c r="P14" s="66"/>
       <x:c r="Q14" s="66"/>
-      <x:c r="R14" s="67" t="str">
-        <x:f>IF($A14="","",IF(COUNT($D14:$Q14)&lt;14,"",ROUND($P14-$D14-($E14-$F14-$G14-$H14-$I14-$J14+$K14+$L14+$M14+$N14-$O14),2)))</x:f>
-      </x:c>
-      <x:c r="S14" s="59" t="str">
-        <x:f>IF($A14="","",IF(DAY($A14)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A14)&gt;1,"Duplicate month",IF(OR($B14="",COUNT($D14:$Q14)&lt;14),"Complete required cells",IF($Q14&gt;MAX($P14,0),"Unavailable cash exceeds closing cash",IF($B14="Partial",IF($C14="","Add cutoff date",IF(OR(YEAR($C14)&lt;&gt;YEAR($A14),MONTH($C14)&lt;&gt;MONTH($A14)),"Cutoff must be in month",IF(ABS($R14)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C14&lt;&gt;"","Remove cutoff date",IF(ABS($R14)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T14" s="55"/>
+      <x:c r="R14" s="109" t="str">
+        <x:f>IF($A14="","",IF(COUNT($D14:$O14)&lt;12,"",ROUND($D14+$E14-$F14-$G14-$H14-$I14-$J14+$K14+$L14+$M14+$N14-$O14,2)))</x:f>
+      </x:c>
+      <x:c r="S14" s="109" t="str">
+        <x:f>IF($A14="","",IF(OR($P14="",$R14=""),"",ROUND($P14-$R14,2)))</x:f>
+      </x:c>
+      <x:c r="T14" s="110" t="str">
+        <x:f>IF($A14="","",IF($A13="","No prior row to compare",IF(EDATE($A13,1)&lt;&gt;$A14,"Check month sequence",IF(OR($D14="",$P13=""),"Check opening cash",IF(ABS($D14-$P13)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U14" s="110" t="str">
+        <x:f>IF($A14="","",IF(DAY($A14)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A14)&gt;1,"Duplicate month",IF(OR($B14="",COUNT($D14:$Q14)&lt;14),"Complete required cells",IF($Q14&gt;MAX($P14,0),"Unavailable cash exceeds closing cash",IF($B14="Partial",IF($C14="","Add cutoff date",IF(OR(YEAR($C14)&lt;&gt;YEAR($A14),MONTH($C14)&lt;&gt;MONTH($A14)),"Cutoff must be in month",IF(ABS($S14)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C14&lt;&gt;"","Remove cutoff date",IF(ABS($S14)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V14" s="55"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="61"/>
@@ -1798,13 +1992,19 @@
       <x:c r="O15" s="66"/>
       <x:c r="P15" s="66"/>
       <x:c r="Q15" s="66"/>
-      <x:c r="R15" s="67" t="str">
-        <x:f>IF($A15="","",IF(COUNT($D15:$Q15)&lt;14,"",ROUND($P15-$D15-($E15-$F15-$G15-$H15-$I15-$J15+$K15+$L15+$M15+$N15-$O15),2)))</x:f>
-      </x:c>
-      <x:c r="S15" s="59" t="str">
-        <x:f>IF($A15="","",IF(DAY($A15)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A15)&gt;1,"Duplicate month",IF(OR($B15="",COUNT($D15:$Q15)&lt;14),"Complete required cells",IF($Q15&gt;MAX($P15,0),"Unavailable cash exceeds closing cash",IF($B15="Partial",IF($C15="","Add cutoff date",IF(OR(YEAR($C15)&lt;&gt;YEAR($A15),MONTH($C15)&lt;&gt;MONTH($A15)),"Cutoff must be in month",IF(ABS($R15)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C15&lt;&gt;"","Remove cutoff date",IF(ABS($R15)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T15" s="55"/>
+      <x:c r="R15" s="109" t="str">
+        <x:f>IF($A15="","",IF(COUNT($D15:$O15)&lt;12,"",ROUND($D15+$E15-$F15-$G15-$H15-$I15-$J15+$K15+$L15+$M15+$N15-$O15,2)))</x:f>
+      </x:c>
+      <x:c r="S15" s="109" t="str">
+        <x:f>IF($A15="","",IF(OR($P15="",$R15=""),"",ROUND($P15-$R15,2)))</x:f>
+      </x:c>
+      <x:c r="T15" s="110" t="str">
+        <x:f>IF($A15="","",IF($A14="","No prior row to compare",IF(EDATE($A14,1)&lt;&gt;$A15,"Check month sequence",IF(OR($D15="",$P14=""),"Check opening cash",IF(ABS($D15-$P14)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U15" s="110" t="str">
+        <x:f>IF($A15="","",IF(DAY($A15)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A15)&gt;1,"Duplicate month",IF(OR($B15="",COUNT($D15:$Q15)&lt;14),"Complete required cells",IF($Q15&gt;MAX($P15,0),"Unavailable cash exceeds closing cash",IF($B15="Partial",IF($C15="","Add cutoff date",IF(OR(YEAR($C15)&lt;&gt;YEAR($A15),MONTH($C15)&lt;&gt;MONTH($A15)),"Cutoff must be in month",IF(ABS($S15)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C15&lt;&gt;"","Remove cutoff date",IF(ABS($S15)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V15" s="55"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="61"/>
@@ -1824,13 +2024,19 @@
       <x:c r="O16" s="66"/>
       <x:c r="P16" s="66"/>
       <x:c r="Q16" s="66"/>
-      <x:c r="R16" s="67" t="str">
-        <x:f>IF($A16="","",IF(COUNT($D16:$Q16)&lt;14,"",ROUND($P16-$D16-($E16-$F16-$G16-$H16-$I16-$J16+$K16+$L16+$M16+$N16-$O16),2)))</x:f>
-      </x:c>
-      <x:c r="S16" s="59" t="str">
-        <x:f>IF($A16="","",IF(DAY($A16)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A16)&gt;1,"Duplicate month",IF(OR($B16="",COUNT($D16:$Q16)&lt;14),"Complete required cells",IF($Q16&gt;MAX($P16,0),"Unavailable cash exceeds closing cash",IF($B16="Partial",IF($C16="","Add cutoff date",IF(OR(YEAR($C16)&lt;&gt;YEAR($A16),MONTH($C16)&lt;&gt;MONTH($A16)),"Cutoff must be in month",IF(ABS($R16)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C16&lt;&gt;"","Remove cutoff date",IF(ABS($R16)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T16" s="55"/>
+      <x:c r="R16" s="109" t="str">
+        <x:f>IF($A16="","",IF(COUNT($D16:$O16)&lt;12,"",ROUND($D16+$E16-$F16-$G16-$H16-$I16-$J16+$K16+$L16+$M16+$N16-$O16,2)))</x:f>
+      </x:c>
+      <x:c r="S16" s="109" t="str">
+        <x:f>IF($A16="","",IF(OR($P16="",$R16=""),"",ROUND($P16-$R16,2)))</x:f>
+      </x:c>
+      <x:c r="T16" s="110" t="str">
+        <x:f>IF($A16="","",IF($A15="","No prior row to compare",IF(EDATE($A15,1)&lt;&gt;$A16,"Check month sequence",IF(OR($D16="",$P15=""),"Check opening cash",IF(ABS($D16-$P15)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U16" s="110" t="str">
+        <x:f>IF($A16="","",IF(DAY($A16)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A16)&gt;1,"Duplicate month",IF(OR($B16="",COUNT($D16:$Q16)&lt;14),"Complete required cells",IF($Q16&gt;MAX($P16,0),"Unavailable cash exceeds closing cash",IF($B16="Partial",IF($C16="","Add cutoff date",IF(OR(YEAR($C16)&lt;&gt;YEAR($A16),MONTH($C16)&lt;&gt;MONTH($A16)),"Cutoff must be in month",IF(ABS($S16)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C16&lt;&gt;"","Remove cutoff date",IF(ABS($S16)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V16" s="55"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="61"/>
@@ -1850,13 +2056,19 @@
       <x:c r="O17" s="66"/>
       <x:c r="P17" s="66"/>
       <x:c r="Q17" s="66"/>
-      <x:c r="R17" s="67" t="str">
-        <x:f>IF($A17="","",IF(COUNT($D17:$Q17)&lt;14,"",ROUND($P17-$D17-($E17-$F17-$G17-$H17-$I17-$J17+$K17+$L17+$M17+$N17-$O17),2)))</x:f>
-      </x:c>
-      <x:c r="S17" s="59" t="str">
-        <x:f>IF($A17="","",IF(DAY($A17)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A17)&gt;1,"Duplicate month",IF(OR($B17="",COUNT($D17:$Q17)&lt;14),"Complete required cells",IF($Q17&gt;MAX($P17,0),"Unavailable cash exceeds closing cash",IF($B17="Partial",IF($C17="","Add cutoff date",IF(OR(YEAR($C17)&lt;&gt;YEAR($A17),MONTH($C17)&lt;&gt;MONTH($A17)),"Cutoff must be in month",IF(ABS($R17)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C17&lt;&gt;"","Remove cutoff date",IF(ABS($R17)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T17" s="55"/>
+      <x:c r="R17" s="109" t="str">
+        <x:f>IF($A17="","",IF(COUNT($D17:$O17)&lt;12,"",ROUND($D17+$E17-$F17-$G17-$H17-$I17-$J17+$K17+$L17+$M17+$N17-$O17,2)))</x:f>
+      </x:c>
+      <x:c r="S17" s="109" t="str">
+        <x:f>IF($A17="","",IF(OR($P17="",$R17=""),"",ROUND($P17-$R17,2)))</x:f>
+      </x:c>
+      <x:c r="T17" s="110" t="str">
+        <x:f>IF($A17="","",IF($A16="","No prior row to compare",IF(EDATE($A16,1)&lt;&gt;$A17,"Check month sequence",IF(OR($D17="",$P16=""),"Check opening cash",IF(ABS($D17-$P16)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U17" s="110" t="str">
+        <x:f>IF($A17="","",IF(DAY($A17)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A17)&gt;1,"Duplicate month",IF(OR($B17="",COUNT($D17:$Q17)&lt;14),"Complete required cells",IF($Q17&gt;MAX($P17,0),"Unavailable cash exceeds closing cash",IF($B17="Partial",IF($C17="","Add cutoff date",IF(OR(YEAR($C17)&lt;&gt;YEAR($A17),MONTH($C17)&lt;&gt;MONTH($A17)),"Cutoff must be in month",IF(ABS($S17)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C17&lt;&gt;"","Remove cutoff date",IF(ABS($S17)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V17" s="55"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="61"/>
@@ -1876,13 +2088,19 @@
       <x:c r="O18" s="66"/>
       <x:c r="P18" s="66"/>
       <x:c r="Q18" s="66"/>
-      <x:c r="R18" s="67" t="str">
-        <x:f>IF($A18="","",IF(COUNT($D18:$Q18)&lt;14,"",ROUND($P18-$D18-($E18-$F18-$G18-$H18-$I18-$J18+$K18+$L18+$M18+$N18-$O18),2)))</x:f>
-      </x:c>
-      <x:c r="S18" s="59" t="str">
-        <x:f>IF($A18="","",IF(DAY($A18)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A18)&gt;1,"Duplicate month",IF(OR($B18="",COUNT($D18:$Q18)&lt;14),"Complete required cells",IF($Q18&gt;MAX($P18,0),"Unavailable cash exceeds closing cash",IF($B18="Partial",IF($C18="","Add cutoff date",IF(OR(YEAR($C18)&lt;&gt;YEAR($A18),MONTH($C18)&lt;&gt;MONTH($A18)),"Cutoff must be in month",IF(ABS($R18)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C18&lt;&gt;"","Remove cutoff date",IF(ABS($R18)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T18" s="55"/>
+      <x:c r="R18" s="109" t="str">
+        <x:f>IF($A18="","",IF(COUNT($D18:$O18)&lt;12,"",ROUND($D18+$E18-$F18-$G18-$H18-$I18-$J18+$K18+$L18+$M18+$N18-$O18,2)))</x:f>
+      </x:c>
+      <x:c r="S18" s="109" t="str">
+        <x:f>IF($A18="","",IF(OR($P18="",$R18=""),"",ROUND($P18-$R18,2)))</x:f>
+      </x:c>
+      <x:c r="T18" s="110" t="str">
+        <x:f>IF($A18="","",IF($A17="","No prior row to compare",IF(EDATE($A17,1)&lt;&gt;$A18,"Check month sequence",IF(OR($D18="",$P17=""),"Check opening cash",IF(ABS($D18-$P17)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U18" s="110" t="str">
+        <x:f>IF($A18="","",IF(DAY($A18)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A18)&gt;1,"Duplicate month",IF(OR($B18="",COUNT($D18:$Q18)&lt;14),"Complete required cells",IF($Q18&gt;MAX($P18,0),"Unavailable cash exceeds closing cash",IF($B18="Partial",IF($C18="","Add cutoff date",IF(OR(YEAR($C18)&lt;&gt;YEAR($A18),MONTH($C18)&lt;&gt;MONTH($A18)),"Cutoff must be in month",IF(ABS($S18)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C18&lt;&gt;"","Remove cutoff date",IF(ABS($S18)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V18" s="55"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="61"/>
@@ -1902,13 +2120,19 @@
       <x:c r="O19" s="66"/>
       <x:c r="P19" s="66"/>
       <x:c r="Q19" s="66"/>
-      <x:c r="R19" s="67" t="str">
-        <x:f>IF($A19="","",IF(COUNT($D19:$Q19)&lt;14,"",ROUND($P19-$D19-($E19-$F19-$G19-$H19-$I19-$J19+$K19+$L19+$M19+$N19-$O19),2)))</x:f>
-      </x:c>
-      <x:c r="S19" s="59" t="str">
-        <x:f>IF($A19="","",IF(DAY($A19)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A19)&gt;1,"Duplicate month",IF(OR($B19="",COUNT($D19:$Q19)&lt;14),"Complete required cells",IF($Q19&gt;MAX($P19,0),"Unavailable cash exceeds closing cash",IF($B19="Partial",IF($C19="","Add cutoff date",IF(OR(YEAR($C19)&lt;&gt;YEAR($A19),MONTH($C19)&lt;&gt;MONTH($A19)),"Cutoff must be in month",IF(ABS($R19)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C19&lt;&gt;"","Remove cutoff date",IF(ABS($R19)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T19" s="55"/>
+      <x:c r="R19" s="109" t="str">
+        <x:f>IF($A19="","",IF(COUNT($D19:$O19)&lt;12,"",ROUND($D19+$E19-$F19-$G19-$H19-$I19-$J19+$K19+$L19+$M19+$N19-$O19,2)))</x:f>
+      </x:c>
+      <x:c r="S19" s="109" t="str">
+        <x:f>IF($A19="","",IF(OR($P19="",$R19=""),"",ROUND($P19-$R19,2)))</x:f>
+      </x:c>
+      <x:c r="T19" s="110" t="str">
+        <x:f>IF($A19="","",IF($A18="","No prior row to compare",IF(EDATE($A18,1)&lt;&gt;$A19,"Check month sequence",IF(OR($D19="",$P18=""),"Check opening cash",IF(ABS($D19-$P18)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U19" s="110" t="str">
+        <x:f>IF($A19="","",IF(DAY($A19)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A19)&gt;1,"Duplicate month",IF(OR($B19="",COUNT($D19:$Q19)&lt;14),"Complete required cells",IF($Q19&gt;MAX($P19,0),"Unavailable cash exceeds closing cash",IF($B19="Partial",IF($C19="","Add cutoff date",IF(OR(YEAR($C19)&lt;&gt;YEAR($A19),MONTH($C19)&lt;&gt;MONTH($A19)),"Cutoff must be in month",IF(ABS($S19)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C19&lt;&gt;"","Remove cutoff date",IF(ABS($S19)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V19" s="55"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="61"/>
@@ -1928,13 +2152,19 @@
       <x:c r="O20" s="66"/>
       <x:c r="P20" s="66"/>
       <x:c r="Q20" s="66"/>
-      <x:c r="R20" s="67" t="str">
-        <x:f>IF($A20="","",IF(COUNT($D20:$Q20)&lt;14,"",ROUND($P20-$D20-($E20-$F20-$G20-$H20-$I20-$J20+$K20+$L20+$M20+$N20-$O20),2)))</x:f>
-      </x:c>
-      <x:c r="S20" s="59" t="str">
-        <x:f>IF($A20="","",IF(DAY($A20)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A20)&gt;1,"Duplicate month",IF(OR($B20="",COUNT($D20:$Q20)&lt;14),"Complete required cells",IF($Q20&gt;MAX($P20,0),"Unavailable cash exceeds closing cash",IF($B20="Partial",IF($C20="","Add cutoff date",IF(OR(YEAR($C20)&lt;&gt;YEAR($A20),MONTH($C20)&lt;&gt;MONTH($A20)),"Cutoff must be in month",IF(ABS($R20)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C20&lt;&gt;"","Remove cutoff date",IF(ABS($R20)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T20" s="55"/>
+      <x:c r="R20" s="109" t="str">
+        <x:f>IF($A20="","",IF(COUNT($D20:$O20)&lt;12,"",ROUND($D20+$E20-$F20-$G20-$H20-$I20-$J20+$K20+$L20+$M20+$N20-$O20,2)))</x:f>
+      </x:c>
+      <x:c r="S20" s="109" t="str">
+        <x:f>IF($A20="","",IF(OR($P20="",$R20=""),"",ROUND($P20-$R20,2)))</x:f>
+      </x:c>
+      <x:c r="T20" s="110" t="str">
+        <x:f>IF($A20="","",IF($A19="","No prior row to compare",IF(EDATE($A19,1)&lt;&gt;$A20,"Check month sequence",IF(OR($D20="",$P19=""),"Check opening cash",IF(ABS($D20-$P19)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U20" s="110" t="str">
+        <x:f>IF($A20="","",IF(DAY($A20)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A20)&gt;1,"Duplicate month",IF(OR($B20="",COUNT($D20:$Q20)&lt;14),"Complete required cells",IF($Q20&gt;MAX($P20,0),"Unavailable cash exceeds closing cash",IF($B20="Partial",IF($C20="","Add cutoff date",IF(OR(YEAR($C20)&lt;&gt;YEAR($A20),MONTH($C20)&lt;&gt;MONTH($A20)),"Cutoff must be in month",IF(ABS($S20)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C20&lt;&gt;"","Remove cutoff date",IF(ABS($S20)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V20" s="55"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="61"/>
@@ -1954,13 +2184,19 @@
       <x:c r="O21" s="66"/>
       <x:c r="P21" s="66"/>
       <x:c r="Q21" s="66"/>
-      <x:c r="R21" s="67" t="str">
-        <x:f>IF($A21="","",IF(COUNT($D21:$Q21)&lt;14,"",ROUND($P21-$D21-($E21-$F21-$G21-$H21-$I21-$J21+$K21+$L21+$M21+$N21-$O21),2)))</x:f>
-      </x:c>
-      <x:c r="S21" s="59" t="str">
-        <x:f>IF($A21="","",IF(DAY($A21)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A21)&gt;1,"Duplicate month",IF(OR($B21="",COUNT($D21:$Q21)&lt;14),"Complete required cells",IF($Q21&gt;MAX($P21,0),"Unavailable cash exceeds closing cash",IF($B21="Partial",IF($C21="","Add cutoff date",IF(OR(YEAR($C21)&lt;&gt;YEAR($A21),MONTH($C21)&lt;&gt;MONTH($A21)),"Cutoff must be in month",IF(ABS($R21)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C21&lt;&gt;"","Remove cutoff date",IF(ABS($R21)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T21" s="55"/>
+      <x:c r="R21" s="109" t="str">
+        <x:f>IF($A21="","",IF(COUNT($D21:$O21)&lt;12,"",ROUND($D21+$E21-$F21-$G21-$H21-$I21-$J21+$K21+$L21+$M21+$N21-$O21,2)))</x:f>
+      </x:c>
+      <x:c r="S21" s="109" t="str">
+        <x:f>IF($A21="","",IF(OR($P21="",$R21=""),"",ROUND($P21-$R21,2)))</x:f>
+      </x:c>
+      <x:c r="T21" s="110" t="str">
+        <x:f>IF($A21="","",IF($A20="","No prior row to compare",IF(EDATE($A20,1)&lt;&gt;$A21,"Check month sequence",IF(OR($D21="",$P20=""),"Check opening cash",IF(ABS($D21-$P20)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U21" s="110" t="str">
+        <x:f>IF($A21="","",IF(DAY($A21)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A21)&gt;1,"Duplicate month",IF(OR($B21="",COUNT($D21:$Q21)&lt;14),"Complete required cells",IF($Q21&gt;MAX($P21,0),"Unavailable cash exceeds closing cash",IF($B21="Partial",IF($C21="","Add cutoff date",IF(OR(YEAR($C21)&lt;&gt;YEAR($A21),MONTH($C21)&lt;&gt;MONTH($A21)),"Cutoff must be in month",IF(ABS($S21)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C21&lt;&gt;"","Remove cutoff date",IF(ABS($S21)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V21" s="55"/>
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="61"/>
@@ -1980,13 +2216,19 @@
       <x:c r="O22" s="66"/>
       <x:c r="P22" s="66"/>
       <x:c r="Q22" s="66"/>
-      <x:c r="R22" s="67" t="str">
-        <x:f>IF($A22="","",IF(COUNT($D22:$Q22)&lt;14,"",ROUND($P22-$D22-($E22-$F22-$G22-$H22-$I22-$J22+$K22+$L22+$M22+$N22-$O22),2)))</x:f>
-      </x:c>
-      <x:c r="S22" s="59" t="str">
-        <x:f>IF($A22="","",IF(DAY($A22)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A22)&gt;1,"Duplicate month",IF(OR($B22="",COUNT($D22:$Q22)&lt;14),"Complete required cells",IF($Q22&gt;MAX($P22,0),"Unavailable cash exceeds closing cash",IF($B22="Partial",IF($C22="","Add cutoff date",IF(OR(YEAR($C22)&lt;&gt;YEAR($A22),MONTH($C22)&lt;&gt;MONTH($A22)),"Cutoff must be in month",IF(ABS($R22)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C22&lt;&gt;"","Remove cutoff date",IF(ABS($R22)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T22" s="55"/>
+      <x:c r="R22" s="109" t="str">
+        <x:f>IF($A22="","",IF(COUNT($D22:$O22)&lt;12,"",ROUND($D22+$E22-$F22-$G22-$H22-$I22-$J22+$K22+$L22+$M22+$N22-$O22,2)))</x:f>
+      </x:c>
+      <x:c r="S22" s="109" t="str">
+        <x:f>IF($A22="","",IF(OR($P22="",$R22=""),"",ROUND($P22-$R22,2)))</x:f>
+      </x:c>
+      <x:c r="T22" s="110" t="str">
+        <x:f>IF($A22="","",IF($A21="","No prior row to compare",IF(EDATE($A21,1)&lt;&gt;$A22,"Check month sequence",IF(OR($D22="",$P21=""),"Check opening cash",IF(ABS($D22-$P21)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U22" s="110" t="str">
+        <x:f>IF($A22="","",IF(DAY($A22)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A22)&gt;1,"Duplicate month",IF(OR($B22="",COUNT($D22:$Q22)&lt;14),"Complete required cells",IF($Q22&gt;MAX($P22,0),"Unavailable cash exceeds closing cash",IF($B22="Partial",IF($C22="","Add cutoff date",IF(OR(YEAR($C22)&lt;&gt;YEAR($A22),MONTH($C22)&lt;&gt;MONTH($A22)),"Cutoff must be in month",IF(ABS($S22)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C22&lt;&gt;"","Remove cutoff date",IF(ABS($S22)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V22" s="55"/>
     </x:row>
     <x:row r="23">
       <x:c r="A23" s="61"/>
@@ -2006,13 +2248,19 @@
       <x:c r="O23" s="66"/>
       <x:c r="P23" s="66"/>
       <x:c r="Q23" s="66"/>
-      <x:c r="R23" s="67" t="str">
-        <x:f>IF($A23="","",IF(COUNT($D23:$Q23)&lt;14,"",ROUND($P23-$D23-($E23-$F23-$G23-$H23-$I23-$J23+$K23+$L23+$M23+$N23-$O23),2)))</x:f>
-      </x:c>
-      <x:c r="S23" s="59" t="str">
-        <x:f>IF($A23="","",IF(DAY($A23)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A23)&gt;1,"Duplicate month",IF(OR($B23="",COUNT($D23:$Q23)&lt;14),"Complete required cells",IF($Q23&gt;MAX($P23,0),"Unavailable cash exceeds closing cash",IF($B23="Partial",IF($C23="","Add cutoff date",IF(OR(YEAR($C23)&lt;&gt;YEAR($A23),MONTH($C23)&lt;&gt;MONTH($A23)),"Cutoff must be in month",IF(ABS($R23)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C23&lt;&gt;"","Remove cutoff date",IF(ABS($R23)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T23" s="55"/>
+      <x:c r="R23" s="109" t="str">
+        <x:f>IF($A23="","",IF(COUNT($D23:$O23)&lt;12,"",ROUND($D23+$E23-$F23-$G23-$H23-$I23-$J23+$K23+$L23+$M23+$N23-$O23,2)))</x:f>
+      </x:c>
+      <x:c r="S23" s="109" t="str">
+        <x:f>IF($A23="","",IF(OR($P23="",$R23=""),"",ROUND($P23-$R23,2)))</x:f>
+      </x:c>
+      <x:c r="T23" s="110" t="str">
+        <x:f>IF($A23="","",IF($A22="","No prior row to compare",IF(EDATE($A22,1)&lt;&gt;$A23,"Check month sequence",IF(OR($D23="",$P22=""),"Check opening cash",IF(ABS($D23-$P22)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U23" s="110" t="str">
+        <x:f>IF($A23="","",IF(DAY($A23)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A23)&gt;1,"Duplicate month",IF(OR($B23="",COUNT($D23:$Q23)&lt;14),"Complete required cells",IF($Q23&gt;MAX($P23,0),"Unavailable cash exceeds closing cash",IF($B23="Partial",IF($C23="","Add cutoff date",IF(OR(YEAR($C23)&lt;&gt;YEAR($A23),MONTH($C23)&lt;&gt;MONTH($A23)),"Cutoff must be in month",IF(ABS($S23)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C23&lt;&gt;"","Remove cutoff date",IF(ABS($S23)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V23" s="55"/>
     </x:row>
     <x:row r="24">
       <x:c r="A24" s="61"/>
@@ -2032,13 +2280,19 @@
       <x:c r="O24" s="66"/>
       <x:c r="P24" s="66"/>
       <x:c r="Q24" s="66"/>
-      <x:c r="R24" s="67" t="str">
-        <x:f>IF($A24="","",IF(COUNT($D24:$Q24)&lt;14,"",ROUND($P24-$D24-($E24-$F24-$G24-$H24-$I24-$J24+$K24+$L24+$M24+$N24-$O24),2)))</x:f>
-      </x:c>
-      <x:c r="S24" s="59" t="str">
-        <x:f>IF($A24="","",IF(DAY($A24)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A24)&gt;1,"Duplicate month",IF(OR($B24="",COUNT($D24:$Q24)&lt;14),"Complete required cells",IF($Q24&gt;MAX($P24,0),"Unavailable cash exceeds closing cash",IF($B24="Partial",IF($C24="","Add cutoff date",IF(OR(YEAR($C24)&lt;&gt;YEAR($A24),MONTH($C24)&lt;&gt;MONTH($A24)),"Cutoff must be in month",IF(ABS($R24)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C24&lt;&gt;"","Remove cutoff date",IF(ABS($R24)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T24" s="55"/>
+      <x:c r="R24" s="109" t="str">
+        <x:f>IF($A24="","",IF(COUNT($D24:$O24)&lt;12,"",ROUND($D24+$E24-$F24-$G24-$H24-$I24-$J24+$K24+$L24+$M24+$N24-$O24,2)))</x:f>
+      </x:c>
+      <x:c r="S24" s="109" t="str">
+        <x:f>IF($A24="","",IF(OR($P24="",$R24=""),"",ROUND($P24-$R24,2)))</x:f>
+      </x:c>
+      <x:c r="T24" s="110" t="str">
+        <x:f>IF($A24="","",IF($A23="","No prior row to compare",IF(EDATE($A23,1)&lt;&gt;$A24,"Check month sequence",IF(OR($D24="",$P23=""),"Check opening cash",IF(ABS($D24-$P23)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U24" s="110" t="str">
+        <x:f>IF($A24="","",IF(DAY($A24)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A24)&gt;1,"Duplicate month",IF(OR($B24="",COUNT($D24:$Q24)&lt;14),"Complete required cells",IF($Q24&gt;MAX($P24,0),"Unavailable cash exceeds closing cash",IF($B24="Partial",IF($C24="","Add cutoff date",IF(OR(YEAR($C24)&lt;&gt;YEAR($A24),MONTH($C24)&lt;&gt;MONTH($A24)),"Cutoff must be in month",IF(ABS($S24)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C24&lt;&gt;"","Remove cutoff date",IF(ABS($S24)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V24" s="55"/>
     </x:row>
     <x:row r="25">
       <x:c r="A25" s="61"/>
@@ -2058,13 +2312,19 @@
       <x:c r="O25" s="66"/>
       <x:c r="P25" s="66"/>
       <x:c r="Q25" s="66"/>
-      <x:c r="R25" s="67" t="str">
-        <x:f>IF($A25="","",IF(COUNT($D25:$Q25)&lt;14,"",ROUND($P25-$D25-($E25-$F25-$G25-$H25-$I25-$J25+$K25+$L25+$M25+$N25-$O25),2)))</x:f>
-      </x:c>
-      <x:c r="S25" s="59" t="str">
-        <x:f>IF($A25="","",IF(DAY($A25)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A25)&gt;1,"Duplicate month",IF(OR($B25="",COUNT($D25:$Q25)&lt;14),"Complete required cells",IF($Q25&gt;MAX($P25,0),"Unavailable cash exceeds closing cash",IF($B25="Partial",IF($C25="","Add cutoff date",IF(OR(YEAR($C25)&lt;&gt;YEAR($A25),MONTH($C25)&lt;&gt;MONTH($A25)),"Cutoff must be in month",IF(ABS($R25)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C25&lt;&gt;"","Remove cutoff date",IF(ABS($R25)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T25" s="55"/>
+      <x:c r="R25" s="109" t="str">
+        <x:f>IF($A25="","",IF(COUNT($D25:$O25)&lt;12,"",ROUND($D25+$E25-$F25-$G25-$H25-$I25-$J25+$K25+$L25+$M25+$N25-$O25,2)))</x:f>
+      </x:c>
+      <x:c r="S25" s="109" t="str">
+        <x:f>IF($A25="","",IF(OR($P25="",$R25=""),"",ROUND($P25-$R25,2)))</x:f>
+      </x:c>
+      <x:c r="T25" s="110" t="str">
+        <x:f>IF($A25="","",IF($A24="","No prior row to compare",IF(EDATE($A24,1)&lt;&gt;$A25,"Check month sequence",IF(OR($D25="",$P24=""),"Check opening cash",IF(ABS($D25-$P24)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U25" s="110" t="str">
+        <x:f>IF($A25="","",IF(DAY($A25)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A25)&gt;1,"Duplicate month",IF(OR($B25="",COUNT($D25:$Q25)&lt;14),"Complete required cells",IF($Q25&gt;MAX($P25,0),"Unavailable cash exceeds closing cash",IF($B25="Partial",IF($C25="","Add cutoff date",IF(OR(YEAR($C25)&lt;&gt;YEAR($A25),MONTH($C25)&lt;&gt;MONTH($A25)),"Cutoff must be in month",IF(ABS($S25)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C25&lt;&gt;"","Remove cutoff date",IF(ABS($S25)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V25" s="55"/>
     </x:row>
     <x:row r="26">
       <x:c r="A26" s="61"/>
@@ -2084,13 +2344,19 @@
       <x:c r="O26" s="66"/>
       <x:c r="P26" s="66"/>
       <x:c r="Q26" s="66"/>
-      <x:c r="R26" s="67" t="str">
-        <x:f>IF($A26="","",IF(COUNT($D26:$Q26)&lt;14,"",ROUND($P26-$D26-($E26-$F26-$G26-$H26-$I26-$J26+$K26+$L26+$M26+$N26-$O26),2)))</x:f>
-      </x:c>
-      <x:c r="S26" s="59" t="str">
-        <x:f>IF($A26="","",IF(DAY($A26)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A26)&gt;1,"Duplicate month",IF(OR($B26="",COUNT($D26:$Q26)&lt;14),"Complete required cells",IF($Q26&gt;MAX($P26,0),"Unavailable cash exceeds closing cash",IF($B26="Partial",IF($C26="","Add cutoff date",IF(OR(YEAR($C26)&lt;&gt;YEAR($A26),MONTH($C26)&lt;&gt;MONTH($A26)),"Cutoff must be in month",IF(ABS($R26)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C26&lt;&gt;"","Remove cutoff date",IF(ABS($R26)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T26" s="55"/>
+      <x:c r="R26" s="109" t="str">
+        <x:f>IF($A26="","",IF(COUNT($D26:$O26)&lt;12,"",ROUND($D26+$E26-$F26-$G26-$H26-$I26-$J26+$K26+$L26+$M26+$N26-$O26,2)))</x:f>
+      </x:c>
+      <x:c r="S26" s="109" t="str">
+        <x:f>IF($A26="","",IF(OR($P26="",$R26=""),"",ROUND($P26-$R26,2)))</x:f>
+      </x:c>
+      <x:c r="T26" s="110" t="str">
+        <x:f>IF($A26="","",IF($A25="","No prior row to compare",IF(EDATE($A25,1)&lt;&gt;$A26,"Check month sequence",IF(OR($D26="",$P25=""),"Check opening cash",IF(ABS($D26-$P25)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U26" s="110" t="str">
+        <x:f>IF($A26="","",IF(DAY($A26)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A26)&gt;1,"Duplicate month",IF(OR($B26="",COUNT($D26:$Q26)&lt;14),"Complete required cells",IF($Q26&gt;MAX($P26,0),"Unavailable cash exceeds closing cash",IF($B26="Partial",IF($C26="","Add cutoff date",IF(OR(YEAR($C26)&lt;&gt;YEAR($A26),MONTH($C26)&lt;&gt;MONTH($A26)),"Cutoff must be in month",IF(ABS($S26)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C26&lt;&gt;"","Remove cutoff date",IF(ABS($S26)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V26" s="55"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="61"/>
@@ -2110,13 +2376,19 @@
       <x:c r="O27" s="66"/>
       <x:c r="P27" s="66"/>
       <x:c r="Q27" s="66"/>
-      <x:c r="R27" s="67" t="str">
-        <x:f>IF($A27="","",IF(COUNT($D27:$Q27)&lt;14,"",ROUND($P27-$D27-($E27-$F27-$G27-$H27-$I27-$J27+$K27+$L27+$M27+$N27-$O27),2)))</x:f>
-      </x:c>
-      <x:c r="S27" s="59" t="str">
-        <x:f>IF($A27="","",IF(DAY($A27)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A27)&gt;1,"Duplicate month",IF(OR($B27="",COUNT($D27:$Q27)&lt;14),"Complete required cells",IF($Q27&gt;MAX($P27,0),"Unavailable cash exceeds closing cash",IF($B27="Partial",IF($C27="","Add cutoff date",IF(OR(YEAR($C27)&lt;&gt;YEAR($A27),MONTH($C27)&lt;&gt;MONTH($A27)),"Cutoff must be in month",IF(ABS($R27)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C27&lt;&gt;"","Remove cutoff date",IF(ABS($R27)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T27" s="55"/>
+      <x:c r="R27" s="109" t="str">
+        <x:f>IF($A27="","",IF(COUNT($D27:$O27)&lt;12,"",ROUND($D27+$E27-$F27-$G27-$H27-$I27-$J27+$K27+$L27+$M27+$N27-$O27,2)))</x:f>
+      </x:c>
+      <x:c r="S27" s="109" t="str">
+        <x:f>IF($A27="","",IF(OR($P27="",$R27=""),"",ROUND($P27-$R27,2)))</x:f>
+      </x:c>
+      <x:c r="T27" s="110" t="str">
+        <x:f>IF($A27="","",IF($A26="","No prior row to compare",IF(EDATE($A26,1)&lt;&gt;$A27,"Check month sequence",IF(OR($D27="",$P26=""),"Check opening cash",IF(ABS($D27-$P26)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U27" s="110" t="str">
+        <x:f>IF($A27="","",IF(DAY($A27)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A27)&gt;1,"Duplicate month",IF(OR($B27="",COUNT($D27:$Q27)&lt;14),"Complete required cells",IF($Q27&gt;MAX($P27,0),"Unavailable cash exceeds closing cash",IF($B27="Partial",IF($C27="","Add cutoff date",IF(OR(YEAR($C27)&lt;&gt;YEAR($A27),MONTH($C27)&lt;&gt;MONTH($A27)),"Cutoff must be in month",IF(ABS($S27)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C27&lt;&gt;"","Remove cutoff date",IF(ABS($S27)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V27" s="55"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="61"/>
@@ -2136,13 +2408,19 @@
       <x:c r="O28" s="66"/>
       <x:c r="P28" s="66"/>
       <x:c r="Q28" s="66"/>
-      <x:c r="R28" s="67" t="str">
-        <x:f>IF($A28="","",IF(COUNT($D28:$Q28)&lt;14,"",ROUND($P28-$D28-($E28-$F28-$G28-$H28-$I28-$J28+$K28+$L28+$M28+$N28-$O28),2)))</x:f>
-      </x:c>
-      <x:c r="S28" s="59" t="str">
-        <x:f>IF($A28="","",IF(DAY($A28)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A28)&gt;1,"Duplicate month",IF(OR($B28="",COUNT($D28:$Q28)&lt;14),"Complete required cells",IF($Q28&gt;MAX($P28,0),"Unavailable cash exceeds closing cash",IF($B28="Partial",IF($C28="","Add cutoff date",IF(OR(YEAR($C28)&lt;&gt;YEAR($A28),MONTH($C28)&lt;&gt;MONTH($A28)),"Cutoff must be in month",IF(ABS($R28)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C28&lt;&gt;"","Remove cutoff date",IF(ABS($R28)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T28" s="55"/>
+      <x:c r="R28" s="109" t="str">
+        <x:f>IF($A28="","",IF(COUNT($D28:$O28)&lt;12,"",ROUND($D28+$E28-$F28-$G28-$H28-$I28-$J28+$K28+$L28+$M28+$N28-$O28,2)))</x:f>
+      </x:c>
+      <x:c r="S28" s="109" t="str">
+        <x:f>IF($A28="","",IF(OR($P28="",$R28=""),"",ROUND($P28-$R28,2)))</x:f>
+      </x:c>
+      <x:c r="T28" s="110" t="str">
+        <x:f>IF($A28="","",IF($A27="","No prior row to compare",IF(EDATE($A27,1)&lt;&gt;$A28,"Check month sequence",IF(OR($D28="",$P27=""),"Check opening cash",IF(ABS($D28-$P27)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U28" s="110" t="str">
+        <x:f>IF($A28="","",IF(DAY($A28)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A28)&gt;1,"Duplicate month",IF(OR($B28="",COUNT($D28:$Q28)&lt;14),"Complete required cells",IF($Q28&gt;MAX($P28,0),"Unavailable cash exceeds closing cash",IF($B28="Partial",IF($C28="","Add cutoff date",IF(OR(YEAR($C28)&lt;&gt;YEAR($A28),MONTH($C28)&lt;&gt;MONTH($A28)),"Cutoff must be in month",IF(ABS($S28)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C28&lt;&gt;"","Remove cutoff date",IF(ABS($S28)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V28" s="55"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="61"/>
@@ -2162,13 +2440,19 @@
       <x:c r="O29" s="66"/>
       <x:c r="P29" s="66"/>
       <x:c r="Q29" s="66"/>
-      <x:c r="R29" s="67" t="str">
-        <x:f>IF($A29="","",IF(COUNT($D29:$Q29)&lt;14,"",ROUND($P29-$D29-($E29-$F29-$G29-$H29-$I29-$J29+$K29+$L29+$M29+$N29-$O29),2)))</x:f>
-      </x:c>
-      <x:c r="S29" s="59" t="str">
-        <x:f>IF($A29="","",IF(DAY($A29)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A29)&gt;1,"Duplicate month",IF(OR($B29="",COUNT($D29:$Q29)&lt;14),"Complete required cells",IF($Q29&gt;MAX($P29,0),"Unavailable cash exceeds closing cash",IF($B29="Partial",IF($C29="","Add cutoff date",IF(OR(YEAR($C29)&lt;&gt;YEAR($A29),MONTH($C29)&lt;&gt;MONTH($A29)),"Cutoff must be in month",IF(ABS($R29)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C29&lt;&gt;"","Remove cutoff date",IF(ABS($R29)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T29" s="55"/>
+      <x:c r="R29" s="109" t="str">
+        <x:f>IF($A29="","",IF(COUNT($D29:$O29)&lt;12,"",ROUND($D29+$E29-$F29-$G29-$H29-$I29-$J29+$K29+$L29+$M29+$N29-$O29,2)))</x:f>
+      </x:c>
+      <x:c r="S29" s="109" t="str">
+        <x:f>IF($A29="","",IF(OR($P29="",$R29=""),"",ROUND($P29-$R29,2)))</x:f>
+      </x:c>
+      <x:c r="T29" s="110" t="str">
+        <x:f>IF($A29="","",IF($A28="","No prior row to compare",IF(EDATE($A28,1)&lt;&gt;$A29,"Check month sequence",IF(OR($D29="",$P28=""),"Check opening cash",IF(ABS($D29-$P28)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U29" s="110" t="str">
+        <x:f>IF($A29="","",IF(DAY($A29)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A29)&gt;1,"Duplicate month",IF(OR($B29="",COUNT($D29:$Q29)&lt;14),"Complete required cells",IF($Q29&gt;MAX($P29,0),"Unavailable cash exceeds closing cash",IF($B29="Partial",IF($C29="","Add cutoff date",IF(OR(YEAR($C29)&lt;&gt;YEAR($A29),MONTH($C29)&lt;&gt;MONTH($A29)),"Cutoff must be in month",IF(ABS($S29)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C29&lt;&gt;"","Remove cutoff date",IF(ABS($S29)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V29" s="55"/>
     </x:row>
     <x:row r="30">
       <x:c r="A30" s="61"/>
@@ -2188,13 +2472,19 @@
       <x:c r="O30" s="66"/>
       <x:c r="P30" s="66"/>
       <x:c r="Q30" s="66"/>
-      <x:c r="R30" s="67" t="str">
-        <x:f>IF($A30="","",IF(COUNT($D30:$Q30)&lt;14,"",ROUND($P30-$D30-($E30-$F30-$G30-$H30-$I30-$J30+$K30+$L30+$M30+$N30-$O30),2)))</x:f>
-      </x:c>
-      <x:c r="S30" s="59" t="str">
-        <x:f>IF($A30="","",IF(DAY($A30)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A30)&gt;1,"Duplicate month",IF(OR($B30="",COUNT($D30:$Q30)&lt;14),"Complete required cells",IF($Q30&gt;MAX($P30,0),"Unavailable cash exceeds closing cash",IF($B30="Partial",IF($C30="","Add cutoff date",IF(OR(YEAR($C30)&lt;&gt;YEAR($A30),MONTH($C30)&lt;&gt;MONTH($A30)),"Cutoff must be in month",IF(ABS($R30)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C30&lt;&gt;"","Remove cutoff date",IF(ABS($R30)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T30" s="55"/>
+      <x:c r="R30" s="109" t="str">
+        <x:f>IF($A30="","",IF(COUNT($D30:$O30)&lt;12,"",ROUND($D30+$E30-$F30-$G30-$H30-$I30-$J30+$K30+$L30+$M30+$N30-$O30,2)))</x:f>
+      </x:c>
+      <x:c r="S30" s="109" t="str">
+        <x:f>IF($A30="","",IF(OR($P30="",$R30=""),"",ROUND($P30-$R30,2)))</x:f>
+      </x:c>
+      <x:c r="T30" s="110" t="str">
+        <x:f>IF($A30="","",IF($A29="","No prior row to compare",IF(EDATE($A29,1)&lt;&gt;$A30,"Check month sequence",IF(OR($D30="",$P29=""),"Check opening cash",IF(ABS($D30-$P29)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U30" s="110" t="str">
+        <x:f>IF($A30="","",IF(DAY($A30)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A30)&gt;1,"Duplicate month",IF(OR($B30="",COUNT($D30:$Q30)&lt;14),"Complete required cells",IF($Q30&gt;MAX($P30,0),"Unavailable cash exceeds closing cash",IF($B30="Partial",IF($C30="","Add cutoff date",IF(OR(YEAR($C30)&lt;&gt;YEAR($A30),MONTH($C30)&lt;&gt;MONTH($A30)),"Cutoff must be in month",IF(ABS($S30)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C30&lt;&gt;"","Remove cutoff date",IF(ABS($S30)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V30" s="55"/>
     </x:row>
     <x:row r="31">
       <x:c r="A31" s="61"/>
@@ -2214,13 +2504,19 @@
       <x:c r="O31" s="66"/>
       <x:c r="P31" s="66"/>
       <x:c r="Q31" s="66"/>
-      <x:c r="R31" s="67" t="str">
-        <x:f>IF($A31="","",IF(COUNT($D31:$Q31)&lt;14,"",ROUND($P31-$D31-($E31-$F31-$G31-$H31-$I31-$J31+$K31+$L31+$M31+$N31-$O31),2)))</x:f>
-      </x:c>
-      <x:c r="S31" s="59" t="str">
-        <x:f>IF($A31="","",IF(DAY($A31)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A31)&gt;1,"Duplicate month",IF(OR($B31="",COUNT($D31:$Q31)&lt;14),"Complete required cells",IF($Q31&gt;MAX($P31,0),"Unavailable cash exceeds closing cash",IF($B31="Partial",IF($C31="","Add cutoff date",IF(OR(YEAR($C31)&lt;&gt;YEAR($A31),MONTH($C31)&lt;&gt;MONTH($A31)),"Cutoff must be in month",IF(ABS($R31)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C31&lt;&gt;"","Remove cutoff date",IF(ABS($R31)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T31" s="55"/>
+      <x:c r="R31" s="109" t="str">
+        <x:f>IF($A31="","",IF(COUNT($D31:$O31)&lt;12,"",ROUND($D31+$E31-$F31-$G31-$H31-$I31-$J31+$K31+$L31+$M31+$N31-$O31,2)))</x:f>
+      </x:c>
+      <x:c r="S31" s="109" t="str">
+        <x:f>IF($A31="","",IF(OR($P31="",$R31=""),"",ROUND($P31-$R31,2)))</x:f>
+      </x:c>
+      <x:c r="T31" s="110" t="str">
+        <x:f>IF($A31="","",IF($A30="","No prior row to compare",IF(EDATE($A30,1)&lt;&gt;$A31,"Check month sequence",IF(OR($D31="",$P30=""),"Check opening cash",IF(ABS($D31-$P30)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U31" s="110" t="str">
+        <x:f>IF($A31="","",IF(DAY($A31)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A31)&gt;1,"Duplicate month",IF(OR($B31="",COUNT($D31:$Q31)&lt;14),"Complete required cells",IF($Q31&gt;MAX($P31,0),"Unavailable cash exceeds closing cash",IF($B31="Partial",IF($C31="","Add cutoff date",IF(OR(YEAR($C31)&lt;&gt;YEAR($A31),MONTH($C31)&lt;&gt;MONTH($A31)),"Cutoff must be in month",IF(ABS($S31)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C31&lt;&gt;"","Remove cutoff date",IF(ABS($S31)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V31" s="55"/>
     </x:row>
     <x:row r="32">
       <x:c r="A32" s="61"/>
@@ -2240,13 +2536,19 @@
       <x:c r="O32" s="66"/>
       <x:c r="P32" s="66"/>
       <x:c r="Q32" s="66"/>
-      <x:c r="R32" s="67" t="str">
-        <x:f>IF($A32="","",IF(COUNT($D32:$Q32)&lt;14,"",ROUND($P32-$D32-($E32-$F32-$G32-$H32-$I32-$J32+$K32+$L32+$M32+$N32-$O32),2)))</x:f>
-      </x:c>
-      <x:c r="S32" s="59" t="str">
-        <x:f>IF($A32="","",IF(DAY($A32)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A32)&gt;1,"Duplicate month",IF(OR($B32="",COUNT($D32:$Q32)&lt;14),"Complete required cells",IF($Q32&gt;MAX($P32,0),"Unavailable cash exceeds closing cash",IF($B32="Partial",IF($C32="","Add cutoff date",IF(OR(YEAR($C32)&lt;&gt;YEAR($A32),MONTH($C32)&lt;&gt;MONTH($A32)),"Cutoff must be in month",IF(ABS($R32)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C32&lt;&gt;"","Remove cutoff date",IF(ABS($R32)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T32" s="55"/>
+      <x:c r="R32" s="109" t="str">
+        <x:f>IF($A32="","",IF(COUNT($D32:$O32)&lt;12,"",ROUND($D32+$E32-$F32-$G32-$H32-$I32-$J32+$K32+$L32+$M32+$N32-$O32,2)))</x:f>
+      </x:c>
+      <x:c r="S32" s="109" t="str">
+        <x:f>IF($A32="","",IF(OR($P32="",$R32=""),"",ROUND($P32-$R32,2)))</x:f>
+      </x:c>
+      <x:c r="T32" s="110" t="str">
+        <x:f>IF($A32="","",IF($A31="","No prior row to compare",IF(EDATE($A31,1)&lt;&gt;$A32,"Check month sequence",IF(OR($D32="",$P31=""),"Check opening cash",IF(ABS($D32-$P31)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U32" s="110" t="str">
+        <x:f>IF($A32="","",IF(DAY($A32)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A32)&gt;1,"Duplicate month",IF(OR($B32="",COUNT($D32:$Q32)&lt;14),"Complete required cells",IF($Q32&gt;MAX($P32,0),"Unavailable cash exceeds closing cash",IF($B32="Partial",IF($C32="","Add cutoff date",IF(OR(YEAR($C32)&lt;&gt;YEAR($A32),MONTH($C32)&lt;&gt;MONTH($A32)),"Cutoff must be in month",IF(ABS($S32)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C32&lt;&gt;"","Remove cutoff date",IF(ABS($S32)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V32" s="55"/>
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="61"/>
@@ -2266,13 +2568,19 @@
       <x:c r="O33" s="66"/>
       <x:c r="P33" s="66"/>
       <x:c r="Q33" s="66"/>
-      <x:c r="R33" s="67" t="str">
-        <x:f>IF($A33="","",IF(COUNT($D33:$Q33)&lt;14,"",ROUND($P33-$D33-($E33-$F33-$G33-$H33-$I33-$J33+$K33+$L33+$M33+$N33-$O33),2)))</x:f>
-      </x:c>
-      <x:c r="S33" s="59" t="str">
-        <x:f>IF($A33="","",IF(DAY($A33)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A33)&gt;1,"Duplicate month",IF(OR($B33="",COUNT($D33:$Q33)&lt;14),"Complete required cells",IF($Q33&gt;MAX($P33,0),"Unavailable cash exceeds closing cash",IF($B33="Partial",IF($C33="","Add cutoff date",IF(OR(YEAR($C33)&lt;&gt;YEAR($A33),MONTH($C33)&lt;&gt;MONTH($A33)),"Cutoff must be in month",IF(ABS($R33)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C33&lt;&gt;"","Remove cutoff date",IF(ABS($R33)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T33" s="55"/>
+      <x:c r="R33" s="109" t="str">
+        <x:f>IF($A33="","",IF(COUNT($D33:$O33)&lt;12,"",ROUND($D33+$E33-$F33-$G33-$H33-$I33-$J33+$K33+$L33+$M33+$N33-$O33,2)))</x:f>
+      </x:c>
+      <x:c r="S33" s="109" t="str">
+        <x:f>IF($A33="","",IF(OR($P33="",$R33=""),"",ROUND($P33-$R33,2)))</x:f>
+      </x:c>
+      <x:c r="T33" s="110" t="str">
+        <x:f>IF($A33="","",IF($A32="","No prior row to compare",IF(EDATE($A32,1)&lt;&gt;$A33,"Check month sequence",IF(OR($D33="",$P32=""),"Check opening cash",IF(ABS($D33-$P32)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U33" s="110" t="str">
+        <x:f>IF($A33="","",IF(DAY($A33)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A33)&gt;1,"Duplicate month",IF(OR($B33="",COUNT($D33:$Q33)&lt;14),"Complete required cells",IF($Q33&gt;MAX($P33,0),"Unavailable cash exceeds closing cash",IF($B33="Partial",IF($C33="","Add cutoff date",IF(OR(YEAR($C33)&lt;&gt;YEAR($A33),MONTH($C33)&lt;&gt;MONTH($A33)),"Cutoff must be in month",IF(ABS($S33)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C33&lt;&gt;"","Remove cutoff date",IF(ABS($S33)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V33" s="55"/>
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="61"/>
@@ -2292,13 +2600,19 @@
       <x:c r="O34" s="66"/>
       <x:c r="P34" s="66"/>
       <x:c r="Q34" s="66"/>
-      <x:c r="R34" s="67" t="str">
-        <x:f>IF($A34="","",IF(COUNT($D34:$Q34)&lt;14,"",ROUND($P34-$D34-($E34-$F34-$G34-$H34-$I34-$J34+$K34+$L34+$M34+$N34-$O34),2)))</x:f>
-      </x:c>
-      <x:c r="S34" s="59" t="str">
-        <x:f>IF($A34="","",IF(DAY($A34)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A34)&gt;1,"Duplicate month",IF(OR($B34="",COUNT($D34:$Q34)&lt;14),"Complete required cells",IF($Q34&gt;MAX($P34,0),"Unavailable cash exceeds closing cash",IF($B34="Partial",IF($C34="","Add cutoff date",IF(OR(YEAR($C34)&lt;&gt;YEAR($A34),MONTH($C34)&lt;&gt;MONTH($A34)),"Cutoff must be in month",IF(ABS($R34)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C34&lt;&gt;"","Remove cutoff date",IF(ABS($R34)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T34" s="55"/>
+      <x:c r="R34" s="109" t="str">
+        <x:f>IF($A34="","",IF(COUNT($D34:$O34)&lt;12,"",ROUND($D34+$E34-$F34-$G34-$H34-$I34-$J34+$K34+$L34+$M34+$N34-$O34,2)))</x:f>
+      </x:c>
+      <x:c r="S34" s="109" t="str">
+        <x:f>IF($A34="","",IF(OR($P34="",$R34=""),"",ROUND($P34-$R34,2)))</x:f>
+      </x:c>
+      <x:c r="T34" s="110" t="str">
+        <x:f>IF($A34="","",IF($A33="","No prior row to compare",IF(EDATE($A33,1)&lt;&gt;$A34,"Check month sequence",IF(OR($D34="",$P33=""),"Check opening cash",IF(ABS($D34-$P33)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U34" s="110" t="str">
+        <x:f>IF($A34="","",IF(DAY($A34)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A34)&gt;1,"Duplicate month",IF(OR($B34="",COUNT($D34:$Q34)&lt;14),"Complete required cells",IF($Q34&gt;MAX($P34,0),"Unavailable cash exceeds closing cash",IF($B34="Partial",IF($C34="","Add cutoff date",IF(OR(YEAR($C34)&lt;&gt;YEAR($A34),MONTH($C34)&lt;&gt;MONTH($A34)),"Cutoff must be in month",IF(ABS($S34)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C34&lt;&gt;"","Remove cutoff date",IF(ABS($S34)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V34" s="55"/>
     </x:row>
     <x:row r="35">
       <x:c r="A35" s="61"/>
@@ -2318,13 +2632,19 @@
       <x:c r="O35" s="66"/>
       <x:c r="P35" s="66"/>
       <x:c r="Q35" s="66"/>
-      <x:c r="R35" s="67" t="str">
-        <x:f>IF($A35="","",IF(COUNT($D35:$Q35)&lt;14,"",ROUND($P35-$D35-($E35-$F35-$G35-$H35-$I35-$J35+$K35+$L35+$M35+$N35-$O35),2)))</x:f>
-      </x:c>
-      <x:c r="S35" s="59" t="str">
-        <x:f>IF($A35="","",IF(DAY($A35)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A35)&gt;1,"Duplicate month",IF(OR($B35="",COUNT($D35:$Q35)&lt;14),"Complete required cells",IF($Q35&gt;MAX($P35,0),"Unavailable cash exceeds closing cash",IF($B35="Partial",IF($C35="","Add cutoff date",IF(OR(YEAR($C35)&lt;&gt;YEAR($A35),MONTH($C35)&lt;&gt;MONTH($A35)),"Cutoff must be in month",IF(ABS($R35)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C35&lt;&gt;"","Remove cutoff date",IF(ABS($R35)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T35" s="55"/>
+      <x:c r="R35" s="109" t="str">
+        <x:f>IF($A35="","",IF(COUNT($D35:$O35)&lt;12,"",ROUND($D35+$E35-$F35-$G35-$H35-$I35-$J35+$K35+$L35+$M35+$N35-$O35,2)))</x:f>
+      </x:c>
+      <x:c r="S35" s="109" t="str">
+        <x:f>IF($A35="","",IF(OR($P35="",$R35=""),"",ROUND($P35-$R35,2)))</x:f>
+      </x:c>
+      <x:c r="T35" s="110" t="str">
+        <x:f>IF($A35="","",IF($A34="","No prior row to compare",IF(EDATE($A34,1)&lt;&gt;$A35,"Check month sequence",IF(OR($D35="",$P34=""),"Check opening cash",IF(ABS($D35-$P34)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U35" s="110" t="str">
+        <x:f>IF($A35="","",IF(DAY($A35)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A35)&gt;1,"Duplicate month",IF(OR($B35="",COUNT($D35:$Q35)&lt;14),"Complete required cells",IF($Q35&gt;MAX($P35,0),"Unavailable cash exceeds closing cash",IF($B35="Partial",IF($C35="","Add cutoff date",IF(OR(YEAR($C35)&lt;&gt;YEAR($A35),MONTH($C35)&lt;&gt;MONTH($A35)),"Cutoff must be in month",IF(ABS($S35)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C35&lt;&gt;"","Remove cutoff date",IF(ABS($S35)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V35" s="55"/>
     </x:row>
     <x:row r="36">
       <x:c r="A36" s="61"/>
@@ -2344,13 +2664,19 @@
       <x:c r="O36" s="66"/>
       <x:c r="P36" s="66"/>
       <x:c r="Q36" s="66"/>
-      <x:c r="R36" s="67" t="str">
-        <x:f>IF($A36="","",IF(COUNT($D36:$Q36)&lt;14,"",ROUND($P36-$D36-($E36-$F36-$G36-$H36-$I36-$J36+$K36+$L36+$M36+$N36-$O36),2)))</x:f>
-      </x:c>
-      <x:c r="S36" s="59" t="str">
-        <x:f>IF($A36="","",IF(DAY($A36)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A36)&gt;1,"Duplicate month",IF(OR($B36="",COUNT($D36:$Q36)&lt;14),"Complete required cells",IF($Q36&gt;MAX($P36,0),"Unavailable cash exceeds closing cash",IF($B36="Partial",IF($C36="","Add cutoff date",IF(OR(YEAR($C36)&lt;&gt;YEAR($A36),MONTH($C36)&lt;&gt;MONTH($A36)),"Cutoff must be in month",IF(ABS($R36)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C36&lt;&gt;"","Remove cutoff date",IF(ABS($R36)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T36" s="55"/>
+      <x:c r="R36" s="109" t="str">
+        <x:f>IF($A36="","",IF(COUNT($D36:$O36)&lt;12,"",ROUND($D36+$E36-$F36-$G36-$H36-$I36-$J36+$K36+$L36+$M36+$N36-$O36,2)))</x:f>
+      </x:c>
+      <x:c r="S36" s="109" t="str">
+        <x:f>IF($A36="","",IF(OR($P36="",$R36=""),"",ROUND($P36-$R36,2)))</x:f>
+      </x:c>
+      <x:c r="T36" s="110" t="str">
+        <x:f>IF($A36="","",IF($A35="","No prior row to compare",IF(EDATE($A35,1)&lt;&gt;$A36,"Check month sequence",IF(OR($D36="",$P35=""),"Check opening cash",IF(ABS($D36-$P35)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U36" s="110" t="str">
+        <x:f>IF($A36="","",IF(DAY($A36)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A36)&gt;1,"Duplicate month",IF(OR($B36="",COUNT($D36:$Q36)&lt;14),"Complete required cells",IF($Q36&gt;MAX($P36,0),"Unavailable cash exceeds closing cash",IF($B36="Partial",IF($C36="","Add cutoff date",IF(OR(YEAR($C36)&lt;&gt;YEAR($A36),MONTH($C36)&lt;&gt;MONTH($A36)),"Cutoff must be in month",IF(ABS($S36)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C36&lt;&gt;"","Remove cutoff date",IF(ABS($S36)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V36" s="55"/>
     </x:row>
     <x:row r="37">
       <x:c r="A37" s="61"/>
@@ -2370,13 +2696,19 @@
       <x:c r="O37" s="66"/>
       <x:c r="P37" s="66"/>
       <x:c r="Q37" s="66"/>
-      <x:c r="R37" s="67" t="str">
-        <x:f>IF($A37="","",IF(COUNT($D37:$Q37)&lt;14,"",ROUND($P37-$D37-($E37-$F37-$G37-$H37-$I37-$J37+$K37+$L37+$M37+$N37-$O37),2)))</x:f>
-      </x:c>
-      <x:c r="S37" s="59" t="str">
-        <x:f>IF($A37="","",IF(DAY($A37)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A37)&gt;1,"Duplicate month",IF(OR($B37="",COUNT($D37:$Q37)&lt;14),"Complete required cells",IF($Q37&gt;MAX($P37,0),"Unavailable cash exceeds closing cash",IF($B37="Partial",IF($C37="","Add cutoff date",IF(OR(YEAR($C37)&lt;&gt;YEAR($A37),MONTH($C37)&lt;&gt;MONTH($A37)),"Cutoff must be in month",IF(ABS($R37)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C37&lt;&gt;"","Remove cutoff date",IF(ABS($R37)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T37" s="55"/>
+      <x:c r="R37" s="109" t="str">
+        <x:f>IF($A37="","",IF(COUNT($D37:$O37)&lt;12,"",ROUND($D37+$E37-$F37-$G37-$H37-$I37-$J37+$K37+$L37+$M37+$N37-$O37,2)))</x:f>
+      </x:c>
+      <x:c r="S37" s="109" t="str">
+        <x:f>IF($A37="","",IF(OR($P37="",$R37=""),"",ROUND($P37-$R37,2)))</x:f>
+      </x:c>
+      <x:c r="T37" s="110" t="str">
+        <x:f>IF($A37="","",IF($A36="","No prior row to compare",IF(EDATE($A36,1)&lt;&gt;$A37,"Check month sequence",IF(OR($D37="",$P36=""),"Check opening cash",IF(ABS($D37-$P36)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U37" s="110" t="str">
+        <x:f>IF($A37="","",IF(DAY($A37)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A37)&gt;1,"Duplicate month",IF(OR($B37="",COUNT($D37:$Q37)&lt;14),"Complete required cells",IF($Q37&gt;MAX($P37,0),"Unavailable cash exceeds closing cash",IF($B37="Partial",IF($C37="","Add cutoff date",IF(OR(YEAR($C37)&lt;&gt;YEAR($A37),MONTH($C37)&lt;&gt;MONTH($A37)),"Cutoff must be in month",IF(ABS($S37)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C37&lt;&gt;"","Remove cutoff date",IF(ABS($S37)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V37" s="55"/>
     </x:row>
     <x:row r="38">
       <x:c r="A38" s="61"/>
@@ -2396,13 +2728,19 @@
       <x:c r="O38" s="66"/>
       <x:c r="P38" s="66"/>
       <x:c r="Q38" s="66"/>
-      <x:c r="R38" s="67" t="str">
-        <x:f>IF($A38="","",IF(COUNT($D38:$Q38)&lt;14,"",ROUND($P38-$D38-($E38-$F38-$G38-$H38-$I38-$J38+$K38+$L38+$M38+$N38-$O38),2)))</x:f>
-      </x:c>
-      <x:c r="S38" s="59" t="str">
-        <x:f>IF($A38="","",IF(DAY($A38)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A38)&gt;1,"Duplicate month",IF(OR($B38="",COUNT($D38:$Q38)&lt;14),"Complete required cells",IF($Q38&gt;MAX($P38,0),"Unavailable cash exceeds closing cash",IF($B38="Partial",IF($C38="","Add cutoff date",IF(OR(YEAR($C38)&lt;&gt;YEAR($A38),MONTH($C38)&lt;&gt;MONTH($A38)),"Cutoff must be in month",IF(ABS($R38)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C38&lt;&gt;"","Remove cutoff date",IF(ABS($R38)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T38" s="55"/>
+      <x:c r="R38" s="109" t="str">
+        <x:f>IF($A38="","",IF(COUNT($D38:$O38)&lt;12,"",ROUND($D38+$E38-$F38-$G38-$H38-$I38-$J38+$K38+$L38+$M38+$N38-$O38,2)))</x:f>
+      </x:c>
+      <x:c r="S38" s="109" t="str">
+        <x:f>IF($A38="","",IF(OR($P38="",$R38=""),"",ROUND($P38-$R38,2)))</x:f>
+      </x:c>
+      <x:c r="T38" s="110" t="str">
+        <x:f>IF($A38="","",IF($A37="","No prior row to compare",IF(EDATE($A37,1)&lt;&gt;$A38,"Check month sequence",IF(OR($D38="",$P37=""),"Check opening cash",IF(ABS($D38-$P37)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U38" s="110" t="str">
+        <x:f>IF($A38="","",IF(DAY($A38)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A38)&gt;1,"Duplicate month",IF(OR($B38="",COUNT($D38:$Q38)&lt;14),"Complete required cells",IF($Q38&gt;MAX($P38,0),"Unavailable cash exceeds closing cash",IF($B38="Partial",IF($C38="","Add cutoff date",IF(OR(YEAR($C38)&lt;&gt;YEAR($A38),MONTH($C38)&lt;&gt;MONTH($A38)),"Cutoff must be in month",IF(ABS($S38)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C38&lt;&gt;"","Remove cutoff date",IF(ABS($S38)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V38" s="55"/>
     </x:row>
     <x:row r="39">
       <x:c r="A39" s="61"/>
@@ -2422,13 +2760,19 @@
       <x:c r="O39" s="66"/>
       <x:c r="P39" s="66"/>
       <x:c r="Q39" s="66"/>
-      <x:c r="R39" s="67" t="str">
-        <x:f>IF($A39="","",IF(COUNT($D39:$Q39)&lt;14,"",ROUND($P39-$D39-($E39-$F39-$G39-$H39-$I39-$J39+$K39+$L39+$M39+$N39-$O39),2)))</x:f>
-      </x:c>
-      <x:c r="S39" s="59" t="str">
-        <x:f>IF($A39="","",IF(DAY($A39)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A39)&gt;1,"Duplicate month",IF(OR($B39="",COUNT($D39:$Q39)&lt;14),"Complete required cells",IF($Q39&gt;MAX($P39,0),"Unavailable cash exceeds closing cash",IF($B39="Partial",IF($C39="","Add cutoff date",IF(OR(YEAR($C39)&lt;&gt;YEAR($A39),MONTH($C39)&lt;&gt;MONTH($A39)),"Cutoff must be in month",IF(ABS($R39)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C39&lt;&gt;"","Remove cutoff date",IF(ABS($R39)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T39" s="55"/>
+      <x:c r="R39" s="109" t="str">
+        <x:f>IF($A39="","",IF(COUNT($D39:$O39)&lt;12,"",ROUND($D39+$E39-$F39-$G39-$H39-$I39-$J39+$K39+$L39+$M39+$N39-$O39,2)))</x:f>
+      </x:c>
+      <x:c r="S39" s="109" t="str">
+        <x:f>IF($A39="","",IF(OR($P39="",$R39=""),"",ROUND($P39-$R39,2)))</x:f>
+      </x:c>
+      <x:c r="T39" s="110" t="str">
+        <x:f>IF($A39="","",IF($A38="","No prior row to compare",IF(EDATE($A38,1)&lt;&gt;$A39,"Check month sequence",IF(OR($D39="",$P38=""),"Check opening cash",IF(ABS($D39-$P38)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U39" s="110" t="str">
+        <x:f>IF($A39="","",IF(DAY($A39)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A39)&gt;1,"Duplicate month",IF(OR($B39="",COUNT($D39:$Q39)&lt;14),"Complete required cells",IF($Q39&gt;MAX($P39,0),"Unavailable cash exceeds closing cash",IF($B39="Partial",IF($C39="","Add cutoff date",IF(OR(YEAR($C39)&lt;&gt;YEAR($A39),MONTH($C39)&lt;&gt;MONTH($A39)),"Cutoff must be in month",IF(ABS($S39)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C39&lt;&gt;"","Remove cutoff date",IF(ABS($S39)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V39" s="55"/>
     </x:row>
     <x:row r="40">
       <x:c r="A40" s="61"/>
@@ -2448,13 +2792,19 @@
       <x:c r="O40" s="66"/>
       <x:c r="P40" s="66"/>
       <x:c r="Q40" s="66"/>
-      <x:c r="R40" s="67" t="str">
-        <x:f>IF($A40="","",IF(COUNT($D40:$Q40)&lt;14,"",ROUND($P40-$D40-($E40-$F40-$G40-$H40-$I40-$J40+$K40+$L40+$M40+$N40-$O40),2)))</x:f>
-      </x:c>
-      <x:c r="S40" s="59" t="str">
-        <x:f>IF($A40="","",IF(DAY($A40)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A40)&gt;1,"Duplicate month",IF(OR($B40="",COUNT($D40:$Q40)&lt;14),"Complete required cells",IF($Q40&gt;MAX($P40,0),"Unavailable cash exceeds closing cash",IF($B40="Partial",IF($C40="","Add cutoff date",IF(OR(YEAR($C40)&lt;&gt;YEAR($A40),MONTH($C40)&lt;&gt;MONTH($A40)),"Cutoff must be in month",IF(ABS($R40)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C40&lt;&gt;"","Remove cutoff date",IF(ABS($R40)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T40" s="55"/>
+      <x:c r="R40" s="109" t="str">
+        <x:f>IF($A40="","",IF(COUNT($D40:$O40)&lt;12,"",ROUND($D40+$E40-$F40-$G40-$H40-$I40-$J40+$K40+$L40+$M40+$N40-$O40,2)))</x:f>
+      </x:c>
+      <x:c r="S40" s="109" t="str">
+        <x:f>IF($A40="","",IF(OR($P40="",$R40=""),"",ROUND($P40-$R40,2)))</x:f>
+      </x:c>
+      <x:c r="T40" s="110" t="str">
+        <x:f>IF($A40="","",IF($A39="","No prior row to compare",IF(EDATE($A39,1)&lt;&gt;$A40,"Check month sequence",IF(OR($D40="",$P39=""),"Check opening cash",IF(ABS($D40-$P39)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U40" s="110" t="str">
+        <x:f>IF($A40="","",IF(DAY($A40)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A40)&gt;1,"Duplicate month",IF(OR($B40="",COUNT($D40:$Q40)&lt;14),"Complete required cells",IF($Q40&gt;MAX($P40,0),"Unavailable cash exceeds closing cash",IF($B40="Partial",IF($C40="","Add cutoff date",IF(OR(YEAR($C40)&lt;&gt;YEAR($A40),MONTH($C40)&lt;&gt;MONTH($A40)),"Cutoff must be in month",IF(ABS($S40)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C40&lt;&gt;"","Remove cutoff date",IF(ABS($S40)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V40" s="55"/>
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="61"/>
@@ -2474,13 +2824,19 @@
       <x:c r="O41" s="66"/>
       <x:c r="P41" s="66"/>
       <x:c r="Q41" s="66"/>
-      <x:c r="R41" s="67" t="str">
-        <x:f>IF($A41="","",IF(COUNT($D41:$Q41)&lt;14,"",ROUND($P41-$D41-($E41-$F41-$G41-$H41-$I41-$J41+$K41+$L41+$M41+$N41-$O41),2)))</x:f>
-      </x:c>
-      <x:c r="S41" s="59" t="str">
-        <x:f>IF($A41="","",IF(DAY($A41)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A41)&gt;1,"Duplicate month",IF(OR($B41="",COUNT($D41:$Q41)&lt;14),"Complete required cells",IF($Q41&gt;MAX($P41,0),"Unavailable cash exceeds closing cash",IF($B41="Partial",IF($C41="","Add cutoff date",IF(OR(YEAR($C41)&lt;&gt;YEAR($A41),MONTH($C41)&lt;&gt;MONTH($A41)),"Cutoff must be in month",IF(ABS($R41)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C41&lt;&gt;"","Remove cutoff date",IF(ABS($R41)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T41" s="55"/>
+      <x:c r="R41" s="109" t="str">
+        <x:f>IF($A41="","",IF(COUNT($D41:$O41)&lt;12,"",ROUND($D41+$E41-$F41-$G41-$H41-$I41-$J41+$K41+$L41+$M41+$N41-$O41,2)))</x:f>
+      </x:c>
+      <x:c r="S41" s="109" t="str">
+        <x:f>IF($A41="","",IF(OR($P41="",$R41=""),"",ROUND($P41-$R41,2)))</x:f>
+      </x:c>
+      <x:c r="T41" s="110" t="str">
+        <x:f>IF($A41="","",IF($A40="","No prior row to compare",IF(EDATE($A40,1)&lt;&gt;$A41,"Check month sequence",IF(OR($D41="",$P40=""),"Check opening cash",IF(ABS($D41-$P40)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U41" s="110" t="str">
+        <x:f>IF($A41="","",IF(DAY($A41)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A41)&gt;1,"Duplicate month",IF(OR($B41="",COUNT($D41:$Q41)&lt;14),"Complete required cells",IF($Q41&gt;MAX($P41,0),"Unavailable cash exceeds closing cash",IF($B41="Partial",IF($C41="","Add cutoff date",IF(OR(YEAR($C41)&lt;&gt;YEAR($A41),MONTH($C41)&lt;&gt;MONTH($A41)),"Cutoff must be in month",IF(ABS($S41)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C41&lt;&gt;"","Remove cutoff date",IF(ABS($S41)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V41" s="55"/>
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="61"/>
@@ -2500,21 +2856,27 @@
       <x:c r="O42" s="66"/>
       <x:c r="P42" s="66"/>
       <x:c r="Q42" s="66"/>
-      <x:c r="R42" s="67" t="str">
-        <x:f>IF($A42="","",IF(COUNT($D42:$Q42)&lt;14,"",ROUND($P42-$D42-($E42-$F42-$G42-$H42-$I42-$J42+$K42+$L42+$M42+$N42-$O42),2)))</x:f>
-      </x:c>
-      <x:c r="S42" s="59" t="str">
-        <x:f>IF($A42="","",IF(DAY($A42)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A42)&gt;1,"Duplicate month",IF(OR($B42="",COUNT($D42:$Q42)&lt;14),"Complete required cells",IF($Q42&gt;MAX($P42,0),"Unavailable cash exceeds closing cash",IF($B42="Partial",IF($C42="","Add cutoff date",IF(OR(YEAR($C42)&lt;&gt;YEAR($A42),MONTH($C42)&lt;&gt;MONTH($A42)),"Cutoff must be in month",IF(ABS($R42)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C42&lt;&gt;"","Remove cutoff date",IF(ABS($R42)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
-      </x:c>
-      <x:c r="T42" s="55"/>
+      <x:c r="R42" s="109" t="str">
+        <x:f>IF($A42="","",IF(COUNT($D42:$O42)&lt;12,"",ROUND($D42+$E42-$F42-$G42-$H42-$I42-$J42+$K42+$L42+$M42+$N42-$O42,2)))</x:f>
+      </x:c>
+      <x:c r="S42" s="109" t="str">
+        <x:f>IF($A42="","",IF(OR($P42="",$R42=""),"",ROUND($P42-$R42,2)))</x:f>
+      </x:c>
+      <x:c r="T42" s="110" t="str">
+        <x:f>IF($A42="","",IF($A41="","No prior row to compare",IF(EDATE($A41,1)&lt;&gt;$A42,"Check month sequence",IF(OR($D42="",$P41=""),"Check opening cash",IF(ABS($D42-$P41)&lt;=1,"Matches prior closing","Opening differs from prior closing")))))</x:f>
+      </x:c>
+      <x:c r="U42" s="110" t="str">
+        <x:f>IF($A42="","",IF(DAY($A42)&lt;&gt;1,"Month must start on day 1",IF(COUNTIF($A$7:$A$42,$A42)&gt;1,"Duplicate month",IF(OR($B42="",COUNT($D42:$Q42)&lt;14),"Complete required cells",IF($Q42&gt;MAX($P42,0),"Unavailable cash exceeds closing cash",IF($B42="Partial",IF($C42="","Add cutoff date",IF(OR(YEAR($C42)&lt;&gt;YEAR($A42),MONTH($C42)&lt;&gt;MONTH($A42)),"Cutoff must be in month",IF(ABS($S42)&gt;1,"Cash does not reconcile","Ready to upload"))),IF($C42&lt;&gt;"","Remove cutoff date",IF(ABS($S42)&gt;1,"Cash does not reconcile","Ready to upload"))))))))</x:f>
+      </x:c>
+      <x:c r="V42" s="55"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:T2"/>
-    <x:mergeCell ref="A3:T3"/>
+    <x:mergeCell ref="A1:V2"/>
+    <x:mergeCell ref="A3:V3"/>
     <x:mergeCell ref="A5:C5"/>
     <x:mergeCell ref="D5:Q5"/>
-    <x:mergeCell ref="R5:S5"/>
+    <x:mergeCell ref="R5:U5"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="S7:S42">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="Complete required"/>
@@ -3387,10 +3749,19 @@
         <x:v>Unavailable cash</x:v>
       </x:c>
       <x:c r="R5" s="51" t="str">
+        <x:v>Expected closing cash</x:v>
+      </x:c>
+      <x:c r="S5" s="51" t="str">
         <x:v>Reconciliation difference</x:v>
       </x:c>
-      <x:c r="S5" s="51" t="str">
+      <x:c r="T5" s="51" t="str">
+        <x:v>Opening balance check</x:v>
+      </x:c>
+      <x:c r="U5" s="51" t="str">
         <x:v>Row check</x:v>
+      </x:c>
+      <x:c r="V5" s="51" t="str">
+        <x:v>Notes</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3443,13 +3814,23 @@
       <x:c r="Q6" s="96" t="n">
         <x:v>12000</x:v>
       </x:c>
-      <x:c r="R6" s="99" t="n">
-        <x:f>ROUND(P6-D6-(E6-F6-G6-H6-I6-J6+K6+L6+M6+N6-O6),2)</x:f>
+      <x:c r="R6" s="107" t="n">
+        <x:f>ROUND(D6+E6-F6-G6-H6-I6-J6+K6+L6+M6+N6-O6,2)</x:f>
+        <x:v>110000</x:v>
+      </x:c>
+      <x:c r="S6" s="107" t="n">
+        <x:f>ROUND(P6-R6,2)</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="S6" s="100" t="str">
-        <x:f>IF(ABS(R6)&lt;=1,"Reconciles","Review entries")</x:f>
-        <x:v>Reconciles</x:v>
+      <x:c r="T6" s="108" t="str">
+        <x:v>First entered month</x:v>
+      </x:c>
+      <x:c r="U6" s="108" t="str">
+        <x:f>IF(ABS(S6)&lt;=1,"Ready to upload","Cash does not reconcile")</x:f>
+        <x:v>Ready to upload</x:v>
+      </x:c>
+      <x:c r="V6" s="54" t="str">
+        <x:v>Actual cash confirms the entered activity.</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -3636,36 +4017,64 @@
       <x:c r="R14" s="22"/>
       <x:c r="S14" s="22"/>
     </x:row>
-    <x:row r="15" ht="30" customHeight="1">
-      <x:c r="A15" s="13" t="str">
+    <x:row r="15" ht="38" customHeight="1">
+      <x:c r="A15" s="128" t="str">
         <x:v>Reconciliation</x:v>
       </x:c>
-      <x:c r="B15" s="13"/>
-      <x:c r="C15" s="13"/>
-      <x:c r="D15" s="22" t="str">
-        <x:v>Opening cash plus all classified activity equals closing cash, so the difference is zero.</x:v>
-      </x:c>
-      <x:c r="E15" s="22"/>
-      <x:c r="F15" s="22"/>
-      <x:c r="G15" s="22"/>
-      <x:c r="H15" s="22"/>
-      <x:c r="I15" s="22"/>
-      <x:c r="J15" s="22"/>
-      <x:c r="K15" s="22"/>
-      <x:c r="L15" s="22"/>
-      <x:c r="M15" s="22"/>
-      <x:c r="N15" s="22"/>
-      <x:c r="O15" s="22"/>
-      <x:c r="P15" s="22"/>
-      <x:c r="Q15" s="22"/>
-      <x:c r="R15" s="22"/>
-      <x:c r="S15" s="22"/>
+      <x:c r="B15" s="129"/>
+      <x:c r="C15" s="129"/>
+      <x:c r="D15" s="120" t="str">
+        <x:v>Expected closing cash equals the actual closing balance, so the reconciliation difference is zero.</x:v>
+      </x:c>
+      <x:c r="E15" s="120"/>
+      <x:c r="F15" s="120"/>
+      <x:c r="G15" s="120"/>
+      <x:c r="H15" s="120"/>
+      <x:c r="I15" s="120"/>
+      <x:c r="J15" s="120"/>
+      <x:c r="K15" s="120"/>
+      <x:c r="L15" s="120"/>
+      <x:c r="M15" s="120"/>
+      <x:c r="N15" s="120"/>
+      <x:c r="O15" s="120"/>
+      <x:c r="P15" s="120"/>
+      <x:c r="Q15" s="120"/>
+      <x:c r="R15" s="120"/>
+      <x:c r="S15" s="120"/>
+      <x:c r="T15" s="123"/>
+      <x:c r="U15" s="123"/>
+      <x:c r="V15" s="123"/>
+    </x:row>
+    <x:row r="16" ht="38" customHeight="1">
+      <x:c r="A16" s="132" t="str">
+        <x:v>Opening balance check</x:v>
+      </x:c>
+      <x:c r="B16" s="123"/>
+      <x:c r="C16" s="123"/>
+      <x:c r="D16" s="123" t="str">
+        <x:v>For later rows, the workbook compares opening cash with the prior month's actual closing cash and asks you to review any difference.</x:v>
+      </x:c>
+      <x:c r="E16" s="123"/>
+      <x:c r="F16" s="123"/>
+      <x:c r="G16" s="123"/>
+      <x:c r="H16" s="123"/>
+      <x:c r="I16" s="123"/>
+      <x:c r="J16" s="123"/>
+      <x:c r="K16" s="123"/>
+      <x:c r="L16" s="123"/>
+      <x:c r="M16" s="123"/>
+      <x:c r="N16" s="123"/>
+      <x:c r="O16" s="123"/>
+      <x:c r="P16" s="123"/>
+      <x:c r="Q16" s="123"/>
+      <x:c r="R16" s="123"/>
+      <x:c r="S16" s="123"/>
+      <x:c r="T16" s="123"/>
+      <x:c r="U16" s="123"/>
+      <x:c r="V16" s="123"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:S2"/>
-    <x:mergeCell ref="A3:S3"/>
-    <x:mergeCell ref="A9:S9"/>
     <x:mergeCell ref="A10:C10"/>
     <x:mergeCell ref="D10:S10"/>
     <x:mergeCell ref="A11:C11"/>
@@ -3676,8 +4085,13 @@
     <x:mergeCell ref="D13:S13"/>
     <x:mergeCell ref="A14:C14"/>
     <x:mergeCell ref="D14:S14"/>
+    <x:mergeCell ref="A1:V2"/>
+    <x:mergeCell ref="A3:V3"/>
+    <x:mergeCell ref="A9:V9"/>
     <x:mergeCell ref="A15:C15"/>
-    <x:mergeCell ref="D15:S15"/>
+    <x:mergeCell ref="D15:V15"/>
+    <x:mergeCell ref="A16:C16"/>
+    <x:mergeCell ref="D16:V16"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>